<commit_message>
Add risk-of-bias workbook, R analysis script with tests, spreadsheet checks
- tools/build_rob_workbook.py and the RoB template (protocol Section 15 items,
  derived adequacy column for sensitivity analysis 5); compare_extractions.py
  now also compares two RoB files.
- tools/analysis_ipd.R: registered analysis (protocol Sections 12, 16-18) with a
  run log carrying SHA-256 hashes; assumptions listed in a separate note.
- tools/test_analysis_ipd.py: synthetic-data tests cross-checked against
  statsmodels/scipy and hand formulas; deliberate-breakage check done.
- Tests that open both workbooks in LibreOffice Calc and compare derived columns
  and drop-downs; README statements about verification corrected.
- Merge of the old session branch (12 Oct screening export analysis); HANDOFF
  corrected; Methods draft marks the AI statement as pending.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017BKkAkTLfidWPZV4f6Xm8t
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -559,7 +559,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>数据提取工作簿（模板，草稿）v2026-10-11a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
+          <t>数据提取工作簿（模板，草稿）v2026-10-14a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
         </is>
       </c>
     </row>
@@ -752,10 +752,10 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="54" customHeight="1">
+    <row r="29" ht="72" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>• 灰色列的公式用 Python 的 formulas 库按公式文本计算过（九行虚构的测试数据，覆盖各分支，没有保存）；容器里没有 Excel，也没有 LibreOffice 的 Calc，所以文件没有在 Excel 或 WPS 里打开过，下拉列表和版面实际是否正常没有验证。第一次用时请随便填几行试一下，有问题告诉 Claude。</t>
+          <t>• 灰色列的公式已用三种方式核对：Python 的 formulas 库、独立的 Python 规则、LibreOffice Calc（10 组虚构的测试数据，覆盖各分支，结果一致；空行保持为空）。LibreOffice Calc 能正常打开本文件，所有下拉列表都被识别。**但没有在 Excel 或 WPS 里打开过，版面（列宽、冻结窗格、颜色）也没有人眼检查过。** 第一次用时请随便填几行试一下，有问题告诉 Claude。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Full-text guide: D1-D8 decided, FT_log as formal record (no Rayyan), decision sheet, FT_time_log sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -9,12 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FT_log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPD_requests" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FT_time_log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPD_requests" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -550,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -559,7 +560,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>数据提取工作簿（模板，草稿）v2026-10-11a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
+          <t>数据提取工作簿（模板，草稿）v2026-10-17a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
         </is>
       </c>
     </row>
@@ -654,106 +655,113 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>• FT_log：全文筛选记录（如果不用 Rayyan 的全文筛选功能，就用这张表；用了也可作备份）。详细规则见《全文筛选指南》。</t>
+          <t>• FT_log：全文筛选的正式记录（指南 D4，2026 年 10 月 17 日决定：全文阶段不用 Rayyan）。每位筛选员用自己的一份副本，两人都完成之前互不查看。详细规则见《全文筛选指南》。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Reports、Patients：数据提取。</t>
+          <t>• FT_time_log：全文筛选的时间记录。每次开始和结束都写一行（日期、起止时间、处理的篇数），用来代替 Rayyan 的时间戳日志。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周）。</t>
+          <t>• Reports、Patients：数据提取。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
+          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周）。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>• Duration_calc：时间换算计算器。Lists：下拉列表（请勿改动，改了会影响所有表）。</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>3. 与附录 C 的差异（Claude 的操作化，待三位确认）</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>• A2  '伴随疾病'多选项拆成独立的 Yes/No/NR 列；影像学检查方式拆成 US、Doppler US、CT、MRI 四列。另外加了胰尾扭转、肠梗阻两列，因为协议第 13 节的附加结局列了它们。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="54" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
         </is>
       </c>
     </row>
     <row r="24" ht="54" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>• A4  加了衍生列（灰色）：own_patient（敏感性分析 1）、idx_dur_category（四类，边界见 Rules D2）、thrombocytosis（&gt;450）、primary_outcome（Rules D3）、pub_period（第 16 节的发表时期）。这些是 Claude 对协议第 12、16 节的读法，须三位确认。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
+          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
         </is>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>• A7  Age 的取值：协议写'年，两位小数（月数 ÷ 12）'；未报告填 NR；原文写法另存 age_verbatim。只写'child'或'患儿'而没有具体年龄的，年龄填 NR（见全文指南 D2）。</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>4. 没有验证的事</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="54" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30" ht="54" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>• 灰色列的公式用 Python 的 formulas 库按公式文本计算过（九行虚构的测试数据，覆盖各分支，没有保存）；容器里没有 Excel，也没有 LibreOffice 的 Calc，所以文件没有在 Excel 或 WPS 里打开过，下拉列表和版面实际是否正常没有验证。第一次用时请随便填几行试一下，有问题告诉 Claude。</t>
         </is>
@@ -1008,7 +1016,7 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>仅 Include 时填（待确认，见指南 D1）</t>
+          <t>仅 Include 时填（指南 D1 已决定：宽松加标记）</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -7063,6 +7071,1033 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F303"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>reviewer</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>n_reports</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="62" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Reviewer</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Session start</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Session end</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Reports handled</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>yyyy-mm-dd</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>R1 = 舒俊，R2 = 卞宏强（全文阶段）</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>开始时间 hh:mm（本地时间）</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>结束时间 hh:mm</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>这一段时间处理了多少篇（整数）</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>例如中断原因、遇到的疑问</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="8" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="8" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="8" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="8" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="8" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="8" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="8" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="8" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="8" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="8" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="8" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="8" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="8" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="8" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="8" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="8" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="8" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="8" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="8" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="8" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="8" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="8" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="8" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="8" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="8" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="8" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="8" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="8" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="8" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="8" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="8" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="8" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="8" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="8" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="8" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="8" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="8" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="8" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="8" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="8" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="8" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="8" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="8" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="8" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="8" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="8" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="8" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="8" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="8" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="8" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="8" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="8" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="8" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="8" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="8" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="8" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="8" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="8" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="8" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="8" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="8" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="8" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="8" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="8" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="8" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="8" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="8" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="8" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="8" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="8" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="8" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="8" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="8" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="8" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="8" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="8" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="8" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="8" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="8" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="8" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="8" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="8" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="8" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="8" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="8" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="8" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="8" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="8" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="8" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="8" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="8" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="8" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="8" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="8" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="8" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="8" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="8" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="8" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="8" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="8" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="8" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="8" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="8" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="8" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="8" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="8" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="8" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="8" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="8" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="8" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="8" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="8" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="8" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="8" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="8" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="8" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="8" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="8" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="8" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="8" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="8" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="8" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="8" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="8" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="8" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="8" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="8" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="8" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="8" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="8" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="8" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="8" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="8" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="8" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="8" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="8" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="8" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="8" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="8" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="8" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="8" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="8" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="8" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="8" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="8" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="8" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="8" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="8" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="8" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="8" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="8" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="8" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="8" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="8" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="8" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="8" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="8" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="8" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="8" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="8" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="8" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="8" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="8" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="8" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="8" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="8" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="8" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="8" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B4:B303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
+      <formula1>Lists!$Y$2:$Y$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Integer" error="请填非负整数。" type="whole" errorStyle="warning" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F75B5"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Q803"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -12958,7 +13993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F75B5"/>
@@ -42789,7 +43824,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -44507,7 +45542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007F7F7F"/>
@@ -44818,7 +45853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007F7F7F"/>
@@ -45494,7 +46529,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00BBBBBB"/>

</xml_diff>

<commit_message>
Full-text stage: name corrected to 卞红强; hand-entry rule deleted; displaced spleen and unobtainable full text are excluded
Guide v2026-10-18b, decision sheet, workbook generator and regenerated
workbooks; CLAUDE.md logs the author's decisions.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -971,7 +971,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>R1 = 舒俊，R2 = 卞宏强（全文阶段），Consensus</t>
+          <t>R1 = 舒俊，R2 = 卞红强（全文阶段），Consensus</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -7154,7 +7154,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>R1 = 舒俊，R2 = 卞宏强（全文阶段）</t>
+          <t>R1 = 舒俊，R2 = 卞红强（全文阶段）</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Extraction reviewers named (Jun Shu, Hongqiang Bian; Jun Yang adjudicates; Ji Wang checks): protocol v1.5, amendment note, workbook EX_time_log, compare_extraction script
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -12,10 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FT_time_log" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPD_requests" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX_time_log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPD_requests" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -560,14 +561,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>数据提取工作簿（模板，草稿）v2026-10-17a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
+          <t>数据提取工作簿（模板，草稿）v2026-10-18a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>依据：协议 v1.4（`Systematic review protocol - PROSPERO draft.docx`）附录 C 的提取表和编码规则，以及第 8、12、13、14、16 节。本工作簿只是把协议落成可填写的表，不改变协议。凡超出附录 C 的地方都列在下面'与附录 C 的差异'里，是 Claude 的操作化建议，三位确认后才生效。</t>
+          <t>依据：协议 v1.5（`Systematic review protocol - PROSPERO draft.docx`）附录 C 的提取表和编码规则，以及第 8、12、13、14、16 节。本工作簿只是把协议落成可填写的表，不改变协议。凡超出附录 C 的地方都列在下面'与附录 C 的差异'里，是 Claude 的操作化建议，三位确认后才生效。</t>
         </is>
       </c>
     </row>
@@ -578,10 +579,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>• 每位提取员各用自己的一份副本（文件名建议 extraction_E1.xlsx、extraction_E2.xlsx，共识文件 extraction_consensus.xlsx）。独立提取完成之前，不看对方的文件。</t>
+          <t>• 提取员：E1 = 舒俊，E2 = 卞红强，分歧由杨俊仲裁；Ji Wang 核查两份提取表但不提取（作者 2026 年 10 月 18 日决定，已写入协议 v1.5）。每位提取员各用自己的一份副本（文件名建议 extraction_E1.xlsx、extraction_E2.xlsx，共识文件 extraction_consensus.xlsx）。独立提取完成之前，不看对方的文件。</t>
         </is>
       </c>
     </row>
@@ -641,10 +642,10 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• 两人完成后比较、做共识：Claude 可以另写比较脚本（出分歧清单和 Cohen's kappa）；协议只说'报告主要暴露和主要结局的 kappa'，没有规定连续变量怎么算——建议对时间类别（四类加缺失）和脾脏存活各算一个 kappa，天数另报一致范围（待确认）。</t>
+          <t>• 两人完成后比较、做共识：用 `tools/compare_extraction.py`（`check` 查一份文件的格式和进度，`compare` 比两份文件并出分歧清单）。协议只说'报告主要暴露和主要结局的 kappa'，没有规定连续变量怎么算——脚本对时间类别（四类加缺失）和脾脏存活各算一个 kappa，天数另报一致范围（这是 Claude 的读法，待确认）。</t>
         </is>
       </c>
     </row>
@@ -676,94 +677,955 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周）。</t>
+          <t>• EX_time_log：数据提取的时间记录，和 FT_time_log 一样，每次开始和结束都写一行（日期、起止时间、处理的报告数和录入的患者数）。这是 Claude 的建议，待确认；没有它，电子表格里看不出每份记录是怎么做出来的。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
+          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周）。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>• Duration_calc：时间换算计算器。Lists：下拉列表（请勿改动，改了会影响所有表）。</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>3. 与附录 C 的差异（Claude 的操作化，待三位确认）</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>• A2  '伴随疾病'多选项拆成独立的 Yes/No/NR 列；影像学检查方式拆成 US、Doppler US、CT、MRI 四列。另外加了胰尾扭转、肠梗阻两列，因为协议第 13 节的附加结局列了它们。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="54" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
         </is>
       </c>
     </row>
     <row r="25" ht="54" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>• A4  加了衍生列（灰色）：own_patient（敏感性分析 1）、idx_dur_category（四类，边界见 Rules D2）、thrombocytosis（&gt;450）、primary_outcome（Rules D3）、pub_period（第 16 节的发表时期）。这些是 Claude 对协议第 12、16 节的读法，须三位确认。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
         </is>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
+          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
         </is>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>• A7  Age 的取值：协议写'年，两位小数（月数 ÷ 12）'；未报告填 NR；原文写法另存 age_verbatim。只写'child'或'患儿'而没有具体年龄的，年龄填 NR（见全文指南 D2）。</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>4. 没有验证的事</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="54" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>• 灰色列的公式用 Python 的 formulas 库按公式文本计算过（九行虚构的测试数据，覆盖各分支，没有保存）；容器里没有 Excel，也没有 LibreOffice 的 Calc，所以文件没有在 Excel 或 WPS 里打开过，下拉列表和版面实际是否正常没有验证。第一次用时请随便填几行试一下，有问题告诉 Claude。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00BBBBBB"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AD11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="44" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="40" customWidth="1" min="28" max="28"/>
+    <col width="37" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>yn</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>yn_nr</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>lang</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>ft_lang</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>consecutive</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>aetiology</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>ws_basis</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>presentation</t>
+        </is>
+      </c>
+      <c r="K1" s="17" t="inlineStr">
+        <is>
+          <t>deferred_reason</t>
+        </is>
+      </c>
+      <c r="L1" s="17" t="inlineStr">
+        <is>
+          <t>torsion_awaiting</t>
+        </is>
+      </c>
+      <c r="M1" s="17" t="inlineStr">
+        <is>
+          <t>perfusion</t>
+        </is>
+      </c>
+      <c r="N1" s="17" t="inlineStr">
+        <is>
+          <t>approach</t>
+        </is>
+      </c>
+      <c r="O1" s="17" t="inlineStr">
+        <is>
+          <t>viability</t>
+        </is>
+      </c>
+      <c r="P1" s="17" t="inlineStr">
+        <is>
+          <t>viab_basis</t>
+        </is>
+      </c>
+      <c r="Q1" s="17" t="inlineStr">
+        <is>
+          <t>procedure</t>
+        </is>
+      </c>
+      <c r="R1" s="17" t="inlineStr">
+        <is>
+          <t>fixation</t>
+        </is>
+      </c>
+      <c r="S1" s="17" t="inlineStr">
+        <is>
+          <t>reason_removed</t>
+        </is>
+      </c>
+      <c r="T1" s="17" t="inlineStr">
+        <is>
+          <t>status_fu</t>
+        </is>
+      </c>
+      <c r="U1" s="17" t="inlineStr">
+        <is>
+          <t>dur_category</t>
+        </is>
+      </c>
+      <c r="V1" s="17" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="W1" s="17" t="inlineStr">
+        <is>
+          <t>phrase</t>
+        </is>
+      </c>
+      <c r="X1" s="17" t="inlineStr">
+        <is>
+          <t>extractor</t>
+        </is>
+      </c>
+      <c r="Y1" s="17" t="inlineStr">
+        <is>
+          <t>ft_reviewer</t>
+        </is>
+      </c>
+      <c r="Z1" s="17" t="inlineStr">
+        <is>
+          <t>ft_decision</t>
+        </is>
+      </c>
+      <c r="AA1" s="17" t="inlineStr">
+        <is>
+          <t>ft_reason</t>
+        </is>
+      </c>
+      <c r="AB1" s="17" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="AC1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_final</t>
+        </is>
+      </c>
+      <c r="AD1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_received</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Case report</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Congenital</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Imaging shows ectopic position or mobility</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Acute</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Family declined</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Viable</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Intraoperative</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Detorsion only</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Mesh</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Failure of fixation</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Preserved</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>&lt;=2 d</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>L other language</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Publisher or open access</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Case series</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Acquired</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Operation shows ectopic position or mobility</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Chronic or intermittent</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Observation advised</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Reduced</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Partially non-viable</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Histology</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Splenopexy</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Retroperitoneal or extraperitoneal pouch</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Surgeon's preference</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Partially preserved</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>3-7 d</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Less than 24 hours / a few hours / overnight</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>D no full text</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Library subscription</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Included with IPD</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cohort</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Imaging and operation</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Acute on chronic</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Elective operation scheduled</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Converted</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Non-viable</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Partial splenectomy +/- splenopexy</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Omental wrap</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Lost</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>8-30 d</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>weeks</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Consensus</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Consensus</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Pending IPD</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>E1 non-human</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Interlibrary loan or document delivery</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Narrative only (no individual data)</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Letter</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Named wandering spleen, no detail</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Asymptomatic</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Total splenectomy</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Direct suture</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>&gt;30 d</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>E2 not wandering spleen</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>CNKI or Wanfang</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Not eligible after check</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Review with new patients</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Torsion only, position not stated</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Mass only</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Autotransplantation</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Other (specify)</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>E3 adults only</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Contact author</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>No operation</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>E4 no original patient data</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>E5 not a formal article</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>Not obtained</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>E6 other</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>A aggregate data only</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>N age not confirmed under 18</t>
         </is>
       </c>
     </row>
@@ -8355,7 +9217,7 @@
       </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>E1 / E2 / Consensus</t>
+          <t>E1 = 舒俊，E2 = 卞红强，Consensus</t>
         </is>
       </c>
       <c r="P3" s="7" t="inlineStr">
@@ -14825,7 +15687,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>E1 = 提取员 1，E2 = 提取员 2，Consensus = 共识</t>
+          <t>E1 = 舒俊，E2 = 卞红强，Consensus = 共识</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -43827,6 +44689,1052 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002F75B5"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G303"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>extractor</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>n_reports</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>n_patients</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="62" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Extractor</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Session start</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Session end</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Reports worked on</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Patients entered</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>yyyy-mm-dd</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>E1 = 舒俊，E2 = 卞红强</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>开始时间 hh:mm（本地时间）</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>结束时间 hh:mm</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>这一段时间处理了多少篇报告（整数）</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>这一段时间录入了多少名患者（整数）</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>例如中断原因、遇到的疑问</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="8" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="8" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="8" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="8" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="8" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="8" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="8" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="8" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="8" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="8" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="8" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="8" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="8" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="8" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="8" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="8" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="8" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="8" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="8" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="8" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="8" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="8" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="8" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="8" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="8" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="8" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="8" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="8" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="8" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="8" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="8" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="8" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="8" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="8" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="8" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="8" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="8" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="8" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="8" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="8" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="8" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="8" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="8" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="8" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="8" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="8" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="8" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="8" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="8" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="8" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="8" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="8" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="8" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="8" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="8" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="8" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="8" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="8" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="8" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="8" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="8" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="8" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="8" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="8" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="8" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="8" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="8" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="8" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="8" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="8" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="8" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="8" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="8" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="8" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="8" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="8" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="8" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="8" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="8" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="8" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="8" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="8" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="8" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="8" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="8" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="8" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="8" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="8" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="8" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="8" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="8" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="8" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="8" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="8" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="8" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="8" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="8" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="8" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="8" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="8" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="8" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="8" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="8" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="8" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="8" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="8" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="8" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="8" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="8" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="8" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="8" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="8" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="8" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="8" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="8" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="8" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="8" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="8" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="8" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="8" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="8" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="8" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="8" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="8" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="8" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="8" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="8" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="8" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="8" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="8" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="8" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="8" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="8" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="8" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="8" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="8" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="8" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="8" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="8" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="8" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="8" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="8" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="8" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="8" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="8" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="8" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="8" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="8" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="8" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="8" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="8" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="8" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="8" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="8" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="8" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="8" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="8" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="8" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="8" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="8" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="8" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="8" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="8" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="8" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="8" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="8" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="8" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="8" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B4:B303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
+      <formula1>Lists!$X$2:$X$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Integer" error="请填非负整数。" type="whole" errorStyle="warning" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Integer" error="请填非负整数。" type="whole" errorStyle="warning" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00548235"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -45542,7 +47450,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007F7F7F"/>
@@ -45853,7 +47761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007F7F7F"/>
@@ -46527,858 +48435,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00BBBBBB"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AD11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="36" customWidth="1" min="17" max="17"/>
-    <col width="42" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="44" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="30" customWidth="1" min="27" max="27"/>
-    <col width="40" customWidth="1" min="28" max="28"/>
-    <col width="37" customWidth="1" min="29" max="29"/>
-    <col width="14" customWidth="1" min="30" max="30"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>yn</t>
-        </is>
-      </c>
-      <c r="B1" s="17" t="inlineStr">
-        <is>
-          <t>yn_nr</t>
-        </is>
-      </c>
-      <c r="C1" s="17" t="inlineStr">
-        <is>
-          <t>sex</t>
-        </is>
-      </c>
-      <c r="D1" s="17" t="inlineStr">
-        <is>
-          <t>lang</t>
-        </is>
-      </c>
-      <c r="E1" s="17" t="inlineStr">
-        <is>
-          <t>ft_lang</t>
-        </is>
-      </c>
-      <c r="F1" s="17" t="inlineStr">
-        <is>
-          <t>design</t>
-        </is>
-      </c>
-      <c r="G1" s="17" t="inlineStr">
-        <is>
-          <t>consecutive</t>
-        </is>
-      </c>
-      <c r="H1" s="17" t="inlineStr">
-        <is>
-          <t>aetiology</t>
-        </is>
-      </c>
-      <c r="I1" s="17" t="inlineStr">
-        <is>
-          <t>ws_basis</t>
-        </is>
-      </c>
-      <c r="J1" s="17" t="inlineStr">
-        <is>
-          <t>presentation</t>
-        </is>
-      </c>
-      <c r="K1" s="17" t="inlineStr">
-        <is>
-          <t>deferred_reason</t>
-        </is>
-      </c>
-      <c r="L1" s="17" t="inlineStr">
-        <is>
-          <t>torsion_awaiting</t>
-        </is>
-      </c>
-      <c r="M1" s="17" t="inlineStr">
-        <is>
-          <t>perfusion</t>
-        </is>
-      </c>
-      <c r="N1" s="17" t="inlineStr">
-        <is>
-          <t>approach</t>
-        </is>
-      </c>
-      <c r="O1" s="17" t="inlineStr">
-        <is>
-          <t>viability</t>
-        </is>
-      </c>
-      <c r="P1" s="17" t="inlineStr">
-        <is>
-          <t>viab_basis</t>
-        </is>
-      </c>
-      <c r="Q1" s="17" t="inlineStr">
-        <is>
-          <t>procedure</t>
-        </is>
-      </c>
-      <c r="R1" s="17" t="inlineStr">
-        <is>
-          <t>fixation</t>
-        </is>
-      </c>
-      <c r="S1" s="17" t="inlineStr">
-        <is>
-          <t>reason_removed</t>
-        </is>
-      </c>
-      <c r="T1" s="17" t="inlineStr">
-        <is>
-          <t>status_fu</t>
-        </is>
-      </c>
-      <c r="U1" s="17" t="inlineStr">
-        <is>
-          <t>dur_category</t>
-        </is>
-      </c>
-      <c r="V1" s="17" t="inlineStr">
-        <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="W1" s="17" t="inlineStr">
-        <is>
-          <t>phrase</t>
-        </is>
-      </c>
-      <c r="X1" s="17" t="inlineStr">
-        <is>
-          <t>extractor</t>
-        </is>
-      </c>
-      <c r="Y1" s="17" t="inlineStr">
-        <is>
-          <t>ft_reviewer</t>
-        </is>
-      </c>
-      <c r="Z1" s="17" t="inlineStr">
-        <is>
-          <t>ft_decision</t>
-        </is>
-      </c>
-      <c r="AA1" s="17" t="inlineStr">
-        <is>
-          <t>ft_reason</t>
-        </is>
-      </c>
-      <c r="AB1" s="17" t="inlineStr">
-        <is>
-          <t>route</t>
-        </is>
-      </c>
-      <c r="AC1" s="17" t="inlineStr">
-        <is>
-          <t>ipd_final</t>
-        </is>
-      </c>
-      <c r="AD1" s="17" t="inlineStr">
-        <is>
-          <t>ipd_received</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Case report</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Congenital</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Imaging shows ectopic position or mobility</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Acute</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Family declined</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Viable</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Intraoperative</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Detorsion only</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Mesh</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Failure of fixation</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Preserved</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>&lt;=2 d</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>hours</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>Include</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>L other language</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>Publisher or open access</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Chinese</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Chinese</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Case series</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Acquired</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Operation shows ectopic position or mobility</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Chronic or intermittent</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Observation advised</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Reduced</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Laparoscopic</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Partially non-viable</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Histology</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Splenopexy</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Retroperitoneal or extraperitoneal pouch</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Surgeon's preference</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Partially preserved</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>3-7 d</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>days</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Less than 24 hours / a few hours / overnight</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>E2</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>Exclude</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>D no full text</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Library subscription</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>Included with IPD</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Cohort</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Imaging and operation</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Acute on chronic</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Elective operation scheduled</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Converted</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Non-viable</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Partial splenectomy +/- splenopexy</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Omental wrap</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Lost</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>8-30 d</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>weeks</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Consensus</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Consensus</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>Pending IPD</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>E1 non-human</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>Interlibrary loan or document delivery</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>Narrative only (no individual data)</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Letter</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Named wandering spleen, no detail</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Asymptomatic</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Total splenectomy</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Direct suture</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>&gt;30 d</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>E2 not wandering spleen</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>CNKI or Wanfang</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Not eligible after check</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Review with new patients</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Torsion only, position not stated</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Mass only</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Autotransplantation</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Other (specify)</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>E3 adults only</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Contact author</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>No operation</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>E4 no original patient data</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>E5 not a formal article</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>Not obtained</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>E6 other</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>A aggregate data only</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>N age not confirmed under 18</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Extraction guide (规则、虚构例子、校准做法); workbook README points to it
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -589,187 +589,194 @@
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>• 逐项怎么填、9 条时间换算规则的虚构例子、疑难情形和校准的做法，见《提取操作说明》（`Extraction guide - how to fill the extraction workbook (draft)`）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>• 表头三行：第 1 行是字段代码（分析时用），第 2 行是协议附录 C 的项目名称，第 3 行是填写说明和允许值。数据从第 4 行开始，请不要在表头上方或表头里插行。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>• Reports 表一行一篇报告；Patients 表一行一名患者，用 report_id 对应。report_id 就是 records_deduplicated.ris 里的 WS 编号；本机构 5 例用 OWN（先在 Reports 表里加一行 OWN），患者编号 OWN_P1–OWN_P5。</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>• **空白和 NR 的区别：** 空白 = 还没提取；NR = 报告里没有这项信息（协议：'Record NR when an item is not reported'）。不要用空白表示没报告。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>• 灰色列是公式，不要改，也不要手填。下拉列表的值不在列表里时 Excel 会警告但允许保存；确需例外，请在 Notes 列写明。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>• 灰色列是公式，不要改，也不要手填。下拉列表的值不在列表里时 Excel 会警告但允许保存；确需例外，请在 Notes 列写明。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>• 关键项要记出处（页、表或图）：协议要求；至少主要暴露（时间）和主要结局（脾脏存活）的出处必填。</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>• 时间换算按 Rules 表的 9 条规则；Duration_calc 表只是计算器，处理不了含糊说法和规则 6–9 的判断，最终以人工判断为准。</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>• 本机构病例只录不可识别的信息：不要写姓名、住院号、出生日期、具体日期。已发表报告的患者也不要抄原文里的姓名缩写。</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>• 校准：正式提取前，两位提取员先各自提取同样的 10 篇报告，比较，讨论分歧，必要时改这份表和规则（协议第 14 节）。10 篇建议涵盖中英文、个案和系列、时间写法各异的报告，在全文名单确定后再选。</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="54" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>• 两人完成后比较、做共识：用 `tools/compare_extraction.py`（`check` 查一份文件的格式和进度，`compare` 比两份文件并出分歧清单）。协议只说'报告主要暴露和主要结局的 kappa'，没有规定连续变量怎么算——脚本对时间类别（四类加缺失）和脾脏存活各算一个 kappa，天数另报一致范围（这是 Claude 的读法，待确认）。</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>2. 各表</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>• FT_log：全文筛选的正式记录（指南 D4，2026 年 10 月 17 日决定：全文阶段不用 Rayyan）。每位筛选员用自己的一份副本，两人都完成之前互不查看。详细规则见《全文筛选指南》。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>• FT_time_log：全文筛选的时间记录。每次开始和结束都写一行（日期、起止时间、处理的篇数），用来代替 Rayyan 的时间戳日志。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>• FT_time_log：全文筛选的时间记录。每次开始和结束都写一行（日期、起止时间、处理的篇数），用来代替 Rayyan 的时间戳日志。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>• Reports、Patients：数据提取。</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>• EX_time_log：数据提取的时间记录，和 FT_time_log 一样，每次开始和结束都写一行（日期、起止时间、处理的报告数和录入的患者数）。这是 Claude 的建议，待确认；没有它，电子表格里看不出每份记录是怎么做出来的。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周）。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
+          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周）。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>• Duration_calc：时间换算计算器。Lists：下拉列表（请勿改动，改了会影响所有表）。</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>3. 与附录 C 的差异（Claude 的操作化，待三位确认）</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
         </is>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>• A2  '伴随疾病'多选项拆成独立的 Yes/No/NR 列；影像学检查方式拆成 US、Doppler US、CT、MRI 四列。另外加了胰尾扭转、肠梗阻两列，因为协议第 13 节的附加结局列了它们。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="54" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
         </is>
       </c>
     </row>
     <row r="26" ht="54" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>• A4  加了衍生列（灰色）：own_patient（敏感性分析 1）、idx_dur_category（四类，边界见 Rules D2）、thrombocytosis（&gt;450）、primary_outcome（Rules D3）、pub_period（第 16 节的发表时期）。这些是 Claude 对协议第 12、16 节的读法，须三位确认。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
         </is>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
+          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
         </is>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>• A7  Age 的取值：协议写'年，两位小数（月数 ÷ 12）'；未报告填 NR；原文写法另存 age_verbatim。只写'child'或'患儿'而没有具体年龄的，年龄填 NR（见全文指南 D2）。</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>4. 没有验证的事</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="54" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>• 灰色列的公式用 Python 的 formulas 库按公式文本计算过（九行虚构的测试数据，覆盖各分支，没有保存）；容器里没有 Excel，也没有 LibreOffice 的 Calc，所以文件没有在 Excel 或 WPS 里打开过，下拉列表和版面实际是否正常没有验证。第一次用时请随便填几行试一下，有问题告诉 Claude。</t>
         </is>

</xml_diff>

<commit_message>
Add contact-log columns to IPD_requests; fix narrative-only status matching in finalize_fulltext
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -561,7 +561,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>数据提取工作簿（模板，草稿）v2026-10-18a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
+          <t>数据提取工作簿（模板，草稿）v2026-10-19a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
         </is>
       </c>
     </row>
@@ -691,10 +691,10 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周）。</t>
+          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周；一报告一行）。联系记录列（2026 年 10 月 19 日加入）：第一封的送达结果、论文邮箱之外用过的途径和日期、是否联系上作者、逐次联系的日志，规则见《IPD 索取邮件》第 1、5 节。邮箱地址和退信邮件都不放进这份表。</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AF11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -827,6 +827,8 @@
     <col width="40" customWidth="1" min="28" max="28"/>
     <col width="37" customWidth="1" min="29" max="29"/>
     <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -980,6 +982,16 @@
           <t>ipd_received</t>
         </is>
       </c>
+      <c r="AE1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_delivery</t>
+        </is>
+      </c>
+      <c r="AF1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_reached</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1132,6 +1144,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Not yet sent</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1284,6 +1306,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Sent, no bounce</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -1421,6 +1453,16 @@
           <t>Partial</t>
         </is>
       </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Bounced</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="F5" t="inlineStr">
@@ -1506,6 +1548,11 @@
       <c r="AC5" t="inlineStr">
         <is>
           <t>Not eligible after check</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>No address found</t>
         </is>
       </c>
     </row>
@@ -45746,7 +45793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L303"/>
+  <dimension ref="A1:Q303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -45755,12 +45802,17 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -45796,30 +45848,55 @@
       </c>
       <c r="G1" s="10" t="inlineStr">
         <is>
+          <t>delivery_result</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
           <t>email2_date</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>reply_date</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>other_routes</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>other_route_date</t>
+        </is>
+      </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>author_reached</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>contact_log</t>
+        </is>
+      </c>
+      <c r="N1" s="10" t="inlineStr">
         <is>
           <t>data_received</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="O1" s="10" t="inlineStr">
         <is>
           <t>data_location</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="P1" s="10" t="inlineStr">
         <is>
           <t>final_status</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -45858,30 +45935,55 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
+          <t>Result of the first e-mail</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
           <t>Second e-mail sent</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="I2" s="10" t="inlineStr">
         <is>
           <t>Reply received</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>Other routes used</t>
+        </is>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
+        <is>
+          <t>First use of another route</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="inlineStr">
+        <is>
+          <t>Author reached?</t>
+        </is>
+      </c>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>Contact log</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="inlineStr">
         <is>
           <t>Individual data received</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="O2" s="10" t="inlineStr">
         <is>
           <t>Where the data file is kept</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="P2" s="10" t="inlineStr">
         <is>
           <t>Final status</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -45906,7 +46008,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>论文 / 机构网页 / 其他</t>
+          <t>论文 / 机构网页 / 其他（不要写邮箱本身）</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -45916,1540 +46018,1871 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
+          <t>Not yet sent / Sent, no bounce / Bounced / No address found（退信只记日期和原因，退信邮件不放进仓库）</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
           <t>yyyy-mm-dd（第一封后 4 周）</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>yyyy-mm-dd</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>论文邮箱之外用过的途径，多个用分号：Institution page; Journal editorial office; Colleague; Other（不要写人名）</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>yyyy-mm-dd；第一次走论文邮箱之外的途径的日期</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>Pending / Yes（有回复，或转交方确认已送达）/ No（到期各条途径都试过，既无回复也无送达确认；到期前不填 No）</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>每次联系写一行：yyyy-mm-dd; 发件人缩写; 途径; 结果。不写邮箱地址。</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
         <is>
           <t>Yes / No / Partial</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>不要放进仓库；只写位置说明</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>Pending / Included with IPD / Narrative only / Not eligible after check</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="Q3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
       <c r="H4" s="8" t="n"/>
+      <c r="I4" s="8" t="n"/>
+      <c r="K4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
       <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
+      <c r="K5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
       <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+      <c r="K6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
       <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
       <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
       <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="K9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
       <c r="H10" s="8" t="n"/>
+      <c r="I10" s="8" t="n"/>
+      <c r="K10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
       <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+      <c r="K11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
       <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
+      <c r="K12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+      <c r="K13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+      <c r="K14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+      <c r="K15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
       <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+      <c r="K16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="F17" s="8" t="n"/>
-      <c r="G17" s="8" t="n"/>
       <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+      <c r="K17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="F18" s="8" t="n"/>
-      <c r="G18" s="8" t="n"/>
       <c r="H18" s="8" t="n"/>
+      <c r="I18" s="8" t="n"/>
+      <c r="K18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
       <c r="H19" s="8" t="n"/>
+      <c r="I19" s="8" t="n"/>
+      <c r="K19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="F20" s="8" t="n"/>
-      <c r="G20" s="8" t="n"/>
       <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="n"/>
+      <c r="I21" s="8" t="n"/>
+      <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
+      <c r="K22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
+      <c r="K23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="F24" s="8" t="n"/>
-      <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="K24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+      <c r="K25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="n"/>
       <c r="H26" s="8" t="n"/>
+      <c r="I26" s="8" t="n"/>
+      <c r="K26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="F27" s="8" t="n"/>
-      <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+      <c r="K27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="n"/>
       <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="K28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="F29" s="8" t="n"/>
-      <c r="G29" s="8" t="n"/>
       <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+      <c r="K29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="F30" s="8" t="n"/>
-      <c r="G30" s="8" t="n"/>
       <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+      <c r="K30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="F31" s="8" t="n"/>
-      <c r="G31" s="8" t="n"/>
       <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+      <c r="K31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="F32" s="8" t="n"/>
-      <c r="G32" s="8" t="n"/>
       <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+      <c r="K32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="F33" s="8" t="n"/>
-      <c r="G33" s="8" t="n"/>
       <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="K33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="F34" s="8" t="n"/>
-      <c r="G34" s="8" t="n"/>
       <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+      <c r="K34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="F35" s="8" t="n"/>
-      <c r="G35" s="8" t="n"/>
       <c r="H35" s="8" t="n"/>
+      <c r="I35" s="8" t="n"/>
+      <c r="K35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="F36" s="8" t="n"/>
-      <c r="G36" s="8" t="n"/>
       <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="n"/>
+      <c r="K36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="F37" s="8" t="n"/>
-      <c r="G37" s="8" t="n"/>
       <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+      <c r="K37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="F38" s="8" t="n"/>
-      <c r="G38" s="8" t="n"/>
       <c r="H38" s="8" t="n"/>
+      <c r="I38" s="8" t="n"/>
+      <c r="K38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="F39" s="8" t="n"/>
-      <c r="G39" s="8" t="n"/>
       <c r="H39" s="8" t="n"/>
+      <c r="I39" s="8" t="n"/>
+      <c r="K39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="F40" s="8" t="n"/>
-      <c r="G40" s="8" t="n"/>
       <c r="H40" s="8" t="n"/>
+      <c r="I40" s="8" t="n"/>
+      <c r="K40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="F41" s="8" t="n"/>
-      <c r="G41" s="8" t="n"/>
       <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="K41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="F42" s="8" t="n"/>
-      <c r="G42" s="8" t="n"/>
       <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="F43" s="8" t="n"/>
-      <c r="G43" s="8" t="n"/>
       <c r="H43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
+      <c r="K43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="F44" s="8" t="n"/>
-      <c r="G44" s="8" t="n"/>
       <c r="H44" s="8" t="n"/>
+      <c r="I44" s="8" t="n"/>
+      <c r="K44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="F45" s="8" t="n"/>
-      <c r="G45" s="8" t="n"/>
       <c r="H45" s="8" t="n"/>
+      <c r="I45" s="8" t="n"/>
+      <c r="K45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="F46" s="8" t="n"/>
-      <c r="G46" s="8" t="n"/>
       <c r="H46" s="8" t="n"/>
+      <c r="I46" s="8" t="n"/>
+      <c r="K46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="F47" s="8" t="n"/>
-      <c r="G47" s="8" t="n"/>
       <c r="H47" s="8" t="n"/>
+      <c r="I47" s="8" t="n"/>
+      <c r="K47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="F48" s="8" t="n"/>
-      <c r="G48" s="8" t="n"/>
       <c r="H48" s="8" t="n"/>
+      <c r="I48" s="8" t="n"/>
+      <c r="K48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="F49" s="8" t="n"/>
-      <c r="G49" s="8" t="n"/>
       <c r="H49" s="8" t="n"/>
+      <c r="I49" s="8" t="n"/>
+      <c r="K49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="F50" s="8" t="n"/>
-      <c r="G50" s="8" t="n"/>
       <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="K50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="F51" s="8" t="n"/>
-      <c r="G51" s="8" t="n"/>
       <c r="H51" s="8" t="n"/>
+      <c r="I51" s="8" t="n"/>
+      <c r="K51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="F52" s="8" t="n"/>
-      <c r="G52" s="8" t="n"/>
       <c r="H52" s="8" t="n"/>
+      <c r="I52" s="8" t="n"/>
+      <c r="K52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="F53" s="8" t="n"/>
-      <c r="G53" s="8" t="n"/>
       <c r="H53" s="8" t="n"/>
+      <c r="I53" s="8" t="n"/>
+      <c r="K53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="F54" s="8" t="n"/>
-      <c r="G54" s="8" t="n"/>
       <c r="H54" s="8" t="n"/>
+      <c r="I54" s="8" t="n"/>
+      <c r="K54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="F55" s="8" t="n"/>
-      <c r="G55" s="8" t="n"/>
       <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="K55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="F56" s="8" t="n"/>
-      <c r="G56" s="8" t="n"/>
       <c r="H56" s="8" t="n"/>
+      <c r="I56" s="8" t="n"/>
+      <c r="K56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="F57" s="8" t="n"/>
-      <c r="G57" s="8" t="n"/>
       <c r="H57" s="8" t="n"/>
+      <c r="I57" s="8" t="n"/>
+      <c r="K57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="F58" s="8" t="n"/>
-      <c r="G58" s="8" t="n"/>
       <c r="H58" s="8" t="n"/>
+      <c r="I58" s="8" t="n"/>
+      <c r="K58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="F59" s="8" t="n"/>
-      <c r="G59" s="8" t="n"/>
       <c r="H59" s="8" t="n"/>
+      <c r="I59" s="8" t="n"/>
+      <c r="K59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="F60" s="8" t="n"/>
-      <c r="G60" s="8" t="n"/>
       <c r="H60" s="8" t="n"/>
+      <c r="I60" s="8" t="n"/>
+      <c r="K60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="F61" s="8" t="n"/>
-      <c r="G61" s="8" t="n"/>
       <c r="H61" s="8" t="n"/>
+      <c r="I61" s="8" t="n"/>
+      <c r="K61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="F62" s="8" t="n"/>
-      <c r="G62" s="8" t="n"/>
       <c r="H62" s="8" t="n"/>
+      <c r="I62" s="8" t="n"/>
+      <c r="K62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="F63" s="8" t="n"/>
-      <c r="G63" s="8" t="n"/>
       <c r="H63" s="8" t="n"/>
+      <c r="I63" s="8" t="n"/>
+      <c r="K63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="F64" s="8" t="n"/>
-      <c r="G64" s="8" t="n"/>
       <c r="H64" s="8" t="n"/>
+      <c r="I64" s="8" t="n"/>
+      <c r="K64" s="8" t="n"/>
     </row>
     <row r="65">
       <c r="F65" s="8" t="n"/>
-      <c r="G65" s="8" t="n"/>
       <c r="H65" s="8" t="n"/>
+      <c r="I65" s="8" t="n"/>
+      <c r="K65" s="8" t="n"/>
     </row>
     <row r="66">
       <c r="F66" s="8" t="n"/>
-      <c r="G66" s="8" t="n"/>
       <c r="H66" s="8" t="n"/>
+      <c r="I66" s="8" t="n"/>
+      <c r="K66" s="8" t="n"/>
     </row>
     <row r="67">
       <c r="F67" s="8" t="n"/>
-      <c r="G67" s="8" t="n"/>
       <c r="H67" s="8" t="n"/>
+      <c r="I67" s="8" t="n"/>
+      <c r="K67" s="8" t="n"/>
     </row>
     <row r="68">
       <c r="F68" s="8" t="n"/>
-      <c r="G68" s="8" t="n"/>
       <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="K68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="F69" s="8" t="n"/>
-      <c r="G69" s="8" t="n"/>
       <c r="H69" s="8" t="n"/>
+      <c r="I69" s="8" t="n"/>
+      <c r="K69" s="8" t="n"/>
     </row>
     <row r="70">
       <c r="F70" s="8" t="n"/>
-      <c r="G70" s="8" t="n"/>
       <c r="H70" s="8" t="n"/>
+      <c r="I70" s="8" t="n"/>
+      <c r="K70" s="8" t="n"/>
     </row>
     <row r="71">
       <c r="F71" s="8" t="n"/>
-      <c r="G71" s="8" t="n"/>
       <c r="H71" s="8" t="n"/>
+      <c r="I71" s="8" t="n"/>
+      <c r="K71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="F72" s="8" t="n"/>
-      <c r="G72" s="8" t="n"/>
       <c r="H72" s="8" t="n"/>
+      <c r="I72" s="8" t="n"/>
+      <c r="K72" s="8" t="n"/>
     </row>
     <row r="73">
       <c r="F73" s="8" t="n"/>
-      <c r="G73" s="8" t="n"/>
       <c r="H73" s="8" t="n"/>
+      <c r="I73" s="8" t="n"/>
+      <c r="K73" s="8" t="n"/>
     </row>
     <row r="74">
       <c r="F74" s="8" t="n"/>
-      <c r="G74" s="8" t="n"/>
       <c r="H74" s="8" t="n"/>
+      <c r="I74" s="8" t="n"/>
+      <c r="K74" s="8" t="n"/>
     </row>
     <row r="75">
       <c r="F75" s="8" t="n"/>
-      <c r="G75" s="8" t="n"/>
       <c r="H75" s="8" t="n"/>
+      <c r="I75" s="8" t="n"/>
+      <c r="K75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="F76" s="8" t="n"/>
-      <c r="G76" s="8" t="n"/>
       <c r="H76" s="8" t="n"/>
+      <c r="I76" s="8" t="n"/>
+      <c r="K76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="F77" s="8" t="n"/>
-      <c r="G77" s="8" t="n"/>
       <c r="H77" s="8" t="n"/>
+      <c r="I77" s="8" t="n"/>
+      <c r="K77" s="8" t="n"/>
     </row>
     <row r="78">
       <c r="F78" s="8" t="n"/>
-      <c r="G78" s="8" t="n"/>
       <c r="H78" s="8" t="n"/>
+      <c r="I78" s="8" t="n"/>
+      <c r="K78" s="8" t="n"/>
     </row>
     <row r="79">
       <c r="F79" s="8" t="n"/>
-      <c r="G79" s="8" t="n"/>
       <c r="H79" s="8" t="n"/>
+      <c r="I79" s="8" t="n"/>
+      <c r="K79" s="8" t="n"/>
     </row>
     <row r="80">
       <c r="F80" s="8" t="n"/>
-      <c r="G80" s="8" t="n"/>
       <c r="H80" s="8" t="n"/>
+      <c r="I80" s="8" t="n"/>
+      <c r="K80" s="8" t="n"/>
     </row>
     <row r="81">
       <c r="F81" s="8" t="n"/>
-      <c r="G81" s="8" t="n"/>
       <c r="H81" s="8" t="n"/>
+      <c r="I81" s="8" t="n"/>
+      <c r="K81" s="8" t="n"/>
     </row>
     <row r="82">
       <c r="F82" s="8" t="n"/>
-      <c r="G82" s="8" t="n"/>
       <c r="H82" s="8" t="n"/>
+      <c r="I82" s="8" t="n"/>
+      <c r="K82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="F83" s="8" t="n"/>
-      <c r="G83" s="8" t="n"/>
       <c r="H83" s="8" t="n"/>
+      <c r="I83" s="8" t="n"/>
+      <c r="K83" s="8" t="n"/>
     </row>
     <row r="84">
       <c r="F84" s="8" t="n"/>
-      <c r="G84" s="8" t="n"/>
       <c r="H84" s="8" t="n"/>
+      <c r="I84" s="8" t="n"/>
+      <c r="K84" s="8" t="n"/>
     </row>
     <row r="85">
       <c r="F85" s="8" t="n"/>
-      <c r="G85" s="8" t="n"/>
       <c r="H85" s="8" t="n"/>
+      <c r="I85" s="8" t="n"/>
+      <c r="K85" s="8" t="n"/>
     </row>
     <row r="86">
       <c r="F86" s="8" t="n"/>
-      <c r="G86" s="8" t="n"/>
       <c r="H86" s="8" t="n"/>
+      <c r="I86" s="8" t="n"/>
+      <c r="K86" s="8" t="n"/>
     </row>
     <row r="87">
       <c r="F87" s="8" t="n"/>
-      <c r="G87" s="8" t="n"/>
       <c r="H87" s="8" t="n"/>
+      <c r="I87" s="8" t="n"/>
+      <c r="K87" s="8" t="n"/>
     </row>
     <row r="88">
       <c r="F88" s="8" t="n"/>
-      <c r="G88" s="8" t="n"/>
       <c r="H88" s="8" t="n"/>
+      <c r="I88" s="8" t="n"/>
+      <c r="K88" s="8" t="n"/>
     </row>
     <row r="89">
       <c r="F89" s="8" t="n"/>
-      <c r="G89" s="8" t="n"/>
       <c r="H89" s="8" t="n"/>
+      <c r="I89" s="8" t="n"/>
+      <c r="K89" s="8" t="n"/>
     </row>
     <row r="90">
       <c r="F90" s="8" t="n"/>
-      <c r="G90" s="8" t="n"/>
       <c r="H90" s="8" t="n"/>
+      <c r="I90" s="8" t="n"/>
+      <c r="K90" s="8" t="n"/>
     </row>
     <row r="91">
       <c r="F91" s="8" t="n"/>
-      <c r="G91" s="8" t="n"/>
       <c r="H91" s="8" t="n"/>
+      <c r="I91" s="8" t="n"/>
+      <c r="K91" s="8" t="n"/>
     </row>
     <row r="92">
       <c r="F92" s="8" t="n"/>
-      <c r="G92" s="8" t="n"/>
       <c r="H92" s="8" t="n"/>
+      <c r="I92" s="8" t="n"/>
+      <c r="K92" s="8" t="n"/>
     </row>
     <row r="93">
       <c r="F93" s="8" t="n"/>
-      <c r="G93" s="8" t="n"/>
       <c r="H93" s="8" t="n"/>
+      <c r="I93" s="8" t="n"/>
+      <c r="K93" s="8" t="n"/>
     </row>
     <row r="94">
       <c r="F94" s="8" t="n"/>
-      <c r="G94" s="8" t="n"/>
       <c r="H94" s="8" t="n"/>
+      <c r="I94" s="8" t="n"/>
+      <c r="K94" s="8" t="n"/>
     </row>
     <row r="95">
       <c r="F95" s="8" t="n"/>
-      <c r="G95" s="8" t="n"/>
       <c r="H95" s="8" t="n"/>
+      <c r="I95" s="8" t="n"/>
+      <c r="K95" s="8" t="n"/>
     </row>
     <row r="96">
       <c r="F96" s="8" t="n"/>
-      <c r="G96" s="8" t="n"/>
       <c r="H96" s="8" t="n"/>
+      <c r="I96" s="8" t="n"/>
+      <c r="K96" s="8" t="n"/>
     </row>
     <row r="97">
       <c r="F97" s="8" t="n"/>
-      <c r="G97" s="8" t="n"/>
       <c r="H97" s="8" t="n"/>
+      <c r="I97" s="8" t="n"/>
+      <c r="K97" s="8" t="n"/>
     </row>
     <row r="98">
       <c r="F98" s="8" t="n"/>
-      <c r="G98" s="8" t="n"/>
       <c r="H98" s="8" t="n"/>
+      <c r="I98" s="8" t="n"/>
+      <c r="K98" s="8" t="n"/>
     </row>
     <row r="99">
       <c r="F99" s="8" t="n"/>
-      <c r="G99" s="8" t="n"/>
       <c r="H99" s="8" t="n"/>
+      <c r="I99" s="8" t="n"/>
+      <c r="K99" s="8" t="n"/>
     </row>
     <row r="100">
       <c r="F100" s="8" t="n"/>
-      <c r="G100" s="8" t="n"/>
       <c r="H100" s="8" t="n"/>
+      <c r="I100" s="8" t="n"/>
+      <c r="K100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="F101" s="8" t="n"/>
-      <c r="G101" s="8" t="n"/>
       <c r="H101" s="8" t="n"/>
+      <c r="I101" s="8" t="n"/>
+      <c r="K101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="F102" s="8" t="n"/>
-      <c r="G102" s="8" t="n"/>
       <c r="H102" s="8" t="n"/>
+      <c r="I102" s="8" t="n"/>
+      <c r="K102" s="8" t="n"/>
     </row>
     <row r="103">
       <c r="F103" s="8" t="n"/>
-      <c r="G103" s="8" t="n"/>
       <c r="H103" s="8" t="n"/>
+      <c r="I103" s="8" t="n"/>
+      <c r="K103" s="8" t="n"/>
     </row>
     <row r="104">
       <c r="F104" s="8" t="n"/>
-      <c r="G104" s="8" t="n"/>
       <c r="H104" s="8" t="n"/>
+      <c r="I104" s="8" t="n"/>
+      <c r="K104" s="8" t="n"/>
     </row>
     <row r="105">
       <c r="F105" s="8" t="n"/>
-      <c r="G105" s="8" t="n"/>
       <c r="H105" s="8" t="n"/>
+      <c r="I105" s="8" t="n"/>
+      <c r="K105" s="8" t="n"/>
     </row>
     <row r="106">
       <c r="F106" s="8" t="n"/>
-      <c r="G106" s="8" t="n"/>
       <c r="H106" s="8" t="n"/>
+      <c r="I106" s="8" t="n"/>
+      <c r="K106" s="8" t="n"/>
     </row>
     <row r="107">
       <c r="F107" s="8" t="n"/>
-      <c r="G107" s="8" t="n"/>
       <c r="H107" s="8" t="n"/>
+      <c r="I107" s="8" t="n"/>
+      <c r="K107" s="8" t="n"/>
     </row>
     <row r="108">
       <c r="F108" s="8" t="n"/>
-      <c r="G108" s="8" t="n"/>
       <c r="H108" s="8" t="n"/>
+      <c r="I108" s="8" t="n"/>
+      <c r="K108" s="8" t="n"/>
     </row>
     <row r="109">
       <c r="F109" s="8" t="n"/>
-      <c r="G109" s="8" t="n"/>
       <c r="H109" s="8" t="n"/>
+      <c r="I109" s="8" t="n"/>
+      <c r="K109" s="8" t="n"/>
     </row>
     <row r="110">
       <c r="F110" s="8" t="n"/>
-      <c r="G110" s="8" t="n"/>
       <c r="H110" s="8" t="n"/>
+      <c r="I110" s="8" t="n"/>
+      <c r="K110" s="8" t="n"/>
     </row>
     <row r="111">
       <c r="F111" s="8" t="n"/>
-      <c r="G111" s="8" t="n"/>
       <c r="H111" s="8" t="n"/>
+      <c r="I111" s="8" t="n"/>
+      <c r="K111" s="8" t="n"/>
     </row>
     <row r="112">
       <c r="F112" s="8" t="n"/>
-      <c r="G112" s="8" t="n"/>
       <c r="H112" s="8" t="n"/>
+      <c r="I112" s="8" t="n"/>
+      <c r="K112" s="8" t="n"/>
     </row>
     <row r="113">
       <c r="F113" s="8" t="n"/>
-      <c r="G113" s="8" t="n"/>
       <c r="H113" s="8" t="n"/>
+      <c r="I113" s="8" t="n"/>
+      <c r="K113" s="8" t="n"/>
     </row>
     <row r="114">
       <c r="F114" s="8" t="n"/>
-      <c r="G114" s="8" t="n"/>
       <c r="H114" s="8" t="n"/>
+      <c r="I114" s="8" t="n"/>
+      <c r="K114" s="8" t="n"/>
     </row>
     <row r="115">
       <c r="F115" s="8" t="n"/>
-      <c r="G115" s="8" t="n"/>
       <c r="H115" s="8" t="n"/>
+      <c r="I115" s="8" t="n"/>
+      <c r="K115" s="8" t="n"/>
     </row>
     <row r="116">
       <c r="F116" s="8" t="n"/>
-      <c r="G116" s="8" t="n"/>
       <c r="H116" s="8" t="n"/>
+      <c r="I116" s="8" t="n"/>
+      <c r="K116" s="8" t="n"/>
     </row>
     <row r="117">
       <c r="F117" s="8" t="n"/>
-      <c r="G117" s="8" t="n"/>
       <c r="H117" s="8" t="n"/>
+      <c r="I117" s="8" t="n"/>
+      <c r="K117" s="8" t="n"/>
     </row>
     <row r="118">
       <c r="F118" s="8" t="n"/>
-      <c r="G118" s="8" t="n"/>
       <c r="H118" s="8" t="n"/>
+      <c r="I118" s="8" t="n"/>
+      <c r="K118" s="8" t="n"/>
     </row>
     <row r="119">
       <c r="F119" s="8" t="n"/>
-      <c r="G119" s="8" t="n"/>
       <c r="H119" s="8" t="n"/>
+      <c r="I119" s="8" t="n"/>
+      <c r="K119" s="8" t="n"/>
     </row>
     <row r="120">
       <c r="F120" s="8" t="n"/>
-      <c r="G120" s="8" t="n"/>
       <c r="H120" s="8" t="n"/>
+      <c r="I120" s="8" t="n"/>
+      <c r="K120" s="8" t="n"/>
     </row>
     <row r="121">
       <c r="F121" s="8" t="n"/>
-      <c r="G121" s="8" t="n"/>
       <c r="H121" s="8" t="n"/>
+      <c r="I121" s="8" t="n"/>
+      <c r="K121" s="8" t="n"/>
     </row>
     <row r="122">
       <c r="F122" s="8" t="n"/>
-      <c r="G122" s="8" t="n"/>
       <c r="H122" s="8" t="n"/>
+      <c r="I122" s="8" t="n"/>
+      <c r="K122" s="8" t="n"/>
     </row>
     <row r="123">
       <c r="F123" s="8" t="n"/>
-      <c r="G123" s="8" t="n"/>
       <c r="H123" s="8" t="n"/>
+      <c r="I123" s="8" t="n"/>
+      <c r="K123" s="8" t="n"/>
     </row>
     <row r="124">
       <c r="F124" s="8" t="n"/>
-      <c r="G124" s="8" t="n"/>
       <c r="H124" s="8" t="n"/>
+      <c r="I124" s="8" t="n"/>
+      <c r="K124" s="8" t="n"/>
     </row>
     <row r="125">
       <c r="F125" s="8" t="n"/>
-      <c r="G125" s="8" t="n"/>
       <c r="H125" s="8" t="n"/>
+      <c r="I125" s="8" t="n"/>
+      <c r="K125" s="8" t="n"/>
     </row>
     <row r="126">
       <c r="F126" s="8" t="n"/>
-      <c r="G126" s="8" t="n"/>
       <c r="H126" s="8" t="n"/>
+      <c r="I126" s="8" t="n"/>
+      <c r="K126" s="8" t="n"/>
     </row>
     <row r="127">
       <c r="F127" s="8" t="n"/>
-      <c r="G127" s="8" t="n"/>
       <c r="H127" s="8" t="n"/>
+      <c r="I127" s="8" t="n"/>
+      <c r="K127" s="8" t="n"/>
     </row>
     <row r="128">
       <c r="F128" s="8" t="n"/>
-      <c r="G128" s="8" t="n"/>
       <c r="H128" s="8" t="n"/>
+      <c r="I128" s="8" t="n"/>
+      <c r="K128" s="8" t="n"/>
     </row>
     <row r="129">
       <c r="F129" s="8" t="n"/>
-      <c r="G129" s="8" t="n"/>
       <c r="H129" s="8" t="n"/>
+      <c r="I129" s="8" t="n"/>
+      <c r="K129" s="8" t="n"/>
     </row>
     <row r="130">
       <c r="F130" s="8" t="n"/>
-      <c r="G130" s="8" t="n"/>
       <c r="H130" s="8" t="n"/>
+      <c r="I130" s="8" t="n"/>
+      <c r="K130" s="8" t="n"/>
     </row>
     <row r="131">
       <c r="F131" s="8" t="n"/>
-      <c r="G131" s="8" t="n"/>
       <c r="H131" s="8" t="n"/>
+      <c r="I131" s="8" t="n"/>
+      <c r="K131" s="8" t="n"/>
     </row>
     <row r="132">
       <c r="F132" s="8" t="n"/>
-      <c r="G132" s="8" t="n"/>
       <c r="H132" s="8" t="n"/>
+      <c r="I132" s="8" t="n"/>
+      <c r="K132" s="8" t="n"/>
     </row>
     <row r="133">
       <c r="F133" s="8" t="n"/>
-      <c r="G133" s="8" t="n"/>
       <c r="H133" s="8" t="n"/>
+      <c r="I133" s="8" t="n"/>
+      <c r="K133" s="8" t="n"/>
     </row>
     <row r="134">
       <c r="F134" s="8" t="n"/>
-      <c r="G134" s="8" t="n"/>
       <c r="H134" s="8" t="n"/>
+      <c r="I134" s="8" t="n"/>
+      <c r="K134" s="8" t="n"/>
     </row>
     <row r="135">
       <c r="F135" s="8" t="n"/>
-      <c r="G135" s="8" t="n"/>
       <c r="H135" s="8" t="n"/>
+      <c r="I135" s="8" t="n"/>
+      <c r="K135" s="8" t="n"/>
     </row>
     <row r="136">
       <c r="F136" s="8" t="n"/>
-      <c r="G136" s="8" t="n"/>
       <c r="H136" s="8" t="n"/>
+      <c r="I136" s="8" t="n"/>
+      <c r="K136" s="8" t="n"/>
     </row>
     <row r="137">
       <c r="F137" s="8" t="n"/>
-      <c r="G137" s="8" t="n"/>
       <c r="H137" s="8" t="n"/>
+      <c r="I137" s="8" t="n"/>
+      <c r="K137" s="8" t="n"/>
     </row>
     <row r="138">
       <c r="F138" s="8" t="n"/>
-      <c r="G138" s="8" t="n"/>
       <c r="H138" s="8" t="n"/>
+      <c r="I138" s="8" t="n"/>
+      <c r="K138" s="8" t="n"/>
     </row>
     <row r="139">
       <c r="F139" s="8" t="n"/>
-      <c r="G139" s="8" t="n"/>
       <c r="H139" s="8" t="n"/>
+      <c r="I139" s="8" t="n"/>
+      <c r="K139" s="8" t="n"/>
     </row>
     <row r="140">
       <c r="F140" s="8" t="n"/>
-      <c r="G140" s="8" t="n"/>
       <c r="H140" s="8" t="n"/>
+      <c r="I140" s="8" t="n"/>
+      <c r="K140" s="8" t="n"/>
     </row>
     <row r="141">
       <c r="F141" s="8" t="n"/>
-      <c r="G141" s="8" t="n"/>
       <c r="H141" s="8" t="n"/>
+      <c r="I141" s="8" t="n"/>
+      <c r="K141" s="8" t="n"/>
     </row>
     <row r="142">
       <c r="F142" s="8" t="n"/>
-      <c r="G142" s="8" t="n"/>
       <c r="H142" s="8" t="n"/>
+      <c r="I142" s="8" t="n"/>
+      <c r="K142" s="8" t="n"/>
     </row>
     <row r="143">
       <c r="F143" s="8" t="n"/>
-      <c r="G143" s="8" t="n"/>
       <c r="H143" s="8" t="n"/>
+      <c r="I143" s="8" t="n"/>
+      <c r="K143" s="8" t="n"/>
     </row>
     <row r="144">
       <c r="F144" s="8" t="n"/>
-      <c r="G144" s="8" t="n"/>
       <c r="H144" s="8" t="n"/>
+      <c r="I144" s="8" t="n"/>
+      <c r="K144" s="8" t="n"/>
     </row>
     <row r="145">
       <c r="F145" s="8" t="n"/>
-      <c r="G145" s="8" t="n"/>
       <c r="H145" s="8" t="n"/>
+      <c r="I145" s="8" t="n"/>
+      <c r="K145" s="8" t="n"/>
     </row>
     <row r="146">
       <c r="F146" s="8" t="n"/>
-      <c r="G146" s="8" t="n"/>
       <c r="H146" s="8" t="n"/>
+      <c r="I146" s="8" t="n"/>
+      <c r="K146" s="8" t="n"/>
     </row>
     <row r="147">
       <c r="F147" s="8" t="n"/>
-      <c r="G147" s="8" t="n"/>
       <c r="H147" s="8" t="n"/>
+      <c r="I147" s="8" t="n"/>
+      <c r="K147" s="8" t="n"/>
     </row>
     <row r="148">
       <c r="F148" s="8" t="n"/>
-      <c r="G148" s="8" t="n"/>
       <c r="H148" s="8" t="n"/>
+      <c r="I148" s="8" t="n"/>
+      <c r="K148" s="8" t="n"/>
     </row>
     <row r="149">
       <c r="F149" s="8" t="n"/>
-      <c r="G149" s="8" t="n"/>
       <c r="H149" s="8" t="n"/>
+      <c r="I149" s="8" t="n"/>
+      <c r="K149" s="8" t="n"/>
     </row>
     <row r="150">
       <c r="F150" s="8" t="n"/>
-      <c r="G150" s="8" t="n"/>
       <c r="H150" s="8" t="n"/>
+      <c r="I150" s="8" t="n"/>
+      <c r="K150" s="8" t="n"/>
     </row>
     <row r="151">
       <c r="F151" s="8" t="n"/>
-      <c r="G151" s="8" t="n"/>
       <c r="H151" s="8" t="n"/>
+      <c r="I151" s="8" t="n"/>
+      <c r="K151" s="8" t="n"/>
     </row>
     <row r="152">
       <c r="F152" s="8" t="n"/>
-      <c r="G152" s="8" t="n"/>
       <c r="H152" s="8" t="n"/>
+      <c r="I152" s="8" t="n"/>
+      <c r="K152" s="8" t="n"/>
     </row>
     <row r="153">
       <c r="F153" s="8" t="n"/>
-      <c r="G153" s="8" t="n"/>
       <c r="H153" s="8" t="n"/>
+      <c r="I153" s="8" t="n"/>
+      <c r="K153" s="8" t="n"/>
     </row>
     <row r="154">
       <c r="F154" s="8" t="n"/>
-      <c r="G154" s="8" t="n"/>
       <c r="H154" s="8" t="n"/>
+      <c r="I154" s="8" t="n"/>
+      <c r="K154" s="8" t="n"/>
     </row>
     <row r="155">
       <c r="F155" s="8" t="n"/>
-      <c r="G155" s="8" t="n"/>
       <c r="H155" s="8" t="n"/>
+      <c r="I155" s="8" t="n"/>
+      <c r="K155" s="8" t="n"/>
     </row>
     <row r="156">
       <c r="F156" s="8" t="n"/>
-      <c r="G156" s="8" t="n"/>
       <c r="H156" s="8" t="n"/>
+      <c r="I156" s="8" t="n"/>
+      <c r="K156" s="8" t="n"/>
     </row>
     <row r="157">
       <c r="F157" s="8" t="n"/>
-      <c r="G157" s="8" t="n"/>
       <c r="H157" s="8" t="n"/>
+      <c r="I157" s="8" t="n"/>
+      <c r="K157" s="8" t="n"/>
     </row>
     <row r="158">
       <c r="F158" s="8" t="n"/>
-      <c r="G158" s="8" t="n"/>
       <c r="H158" s="8" t="n"/>
+      <c r="I158" s="8" t="n"/>
+      <c r="K158" s="8" t="n"/>
     </row>
     <row r="159">
       <c r="F159" s="8" t="n"/>
-      <c r="G159" s="8" t="n"/>
       <c r="H159" s="8" t="n"/>
+      <c r="I159" s="8" t="n"/>
+      <c r="K159" s="8" t="n"/>
     </row>
     <row r="160">
       <c r="F160" s="8" t="n"/>
-      <c r="G160" s="8" t="n"/>
       <c r="H160" s="8" t="n"/>
+      <c r="I160" s="8" t="n"/>
+      <c r="K160" s="8" t="n"/>
     </row>
     <row r="161">
       <c r="F161" s="8" t="n"/>
-      <c r="G161" s="8" t="n"/>
       <c r="H161" s="8" t="n"/>
+      <c r="I161" s="8" t="n"/>
+      <c r="K161" s="8" t="n"/>
     </row>
     <row r="162">
       <c r="F162" s="8" t="n"/>
-      <c r="G162" s="8" t="n"/>
       <c r="H162" s="8" t="n"/>
+      <c r="I162" s="8" t="n"/>
+      <c r="K162" s="8" t="n"/>
     </row>
     <row r="163">
       <c r="F163" s="8" t="n"/>
-      <c r="G163" s="8" t="n"/>
       <c r="H163" s="8" t="n"/>
+      <c r="I163" s="8" t="n"/>
+      <c r="K163" s="8" t="n"/>
     </row>
     <row r="164">
       <c r="F164" s="8" t="n"/>
-      <c r="G164" s="8" t="n"/>
       <c r="H164" s="8" t="n"/>
+      <c r="I164" s="8" t="n"/>
+      <c r="K164" s="8" t="n"/>
     </row>
     <row r="165">
       <c r="F165" s="8" t="n"/>
-      <c r="G165" s="8" t="n"/>
       <c r="H165" s="8" t="n"/>
+      <c r="I165" s="8" t="n"/>
+      <c r="K165" s="8" t="n"/>
     </row>
     <row r="166">
       <c r="F166" s="8" t="n"/>
-      <c r="G166" s="8" t="n"/>
       <c r="H166" s="8" t="n"/>
+      <c r="I166" s="8" t="n"/>
+      <c r="K166" s="8" t="n"/>
     </row>
     <row r="167">
       <c r="F167" s="8" t="n"/>
-      <c r="G167" s="8" t="n"/>
       <c r="H167" s="8" t="n"/>
+      <c r="I167" s="8" t="n"/>
+      <c r="K167" s="8" t="n"/>
     </row>
     <row r="168">
       <c r="F168" s="8" t="n"/>
-      <c r="G168" s="8" t="n"/>
       <c r="H168" s="8" t="n"/>
+      <c r="I168" s="8" t="n"/>
+      <c r="K168" s="8" t="n"/>
     </row>
     <row r="169">
       <c r="F169" s="8" t="n"/>
-      <c r="G169" s="8" t="n"/>
       <c r="H169" s="8" t="n"/>
+      <c r="I169" s="8" t="n"/>
+      <c r="K169" s="8" t="n"/>
     </row>
     <row r="170">
       <c r="F170" s="8" t="n"/>
-      <c r="G170" s="8" t="n"/>
       <c r="H170" s="8" t="n"/>
+      <c r="I170" s="8" t="n"/>
+      <c r="K170" s="8" t="n"/>
     </row>
     <row r="171">
       <c r="F171" s="8" t="n"/>
-      <c r="G171" s="8" t="n"/>
       <c r="H171" s="8" t="n"/>
+      <c r="I171" s="8" t="n"/>
+      <c r="K171" s="8" t="n"/>
     </row>
     <row r="172">
       <c r="F172" s="8" t="n"/>
-      <c r="G172" s="8" t="n"/>
       <c r="H172" s="8" t="n"/>
+      <c r="I172" s="8" t="n"/>
+      <c r="K172" s="8" t="n"/>
     </row>
     <row r="173">
       <c r="F173" s="8" t="n"/>
-      <c r="G173" s="8" t="n"/>
       <c r="H173" s="8" t="n"/>
+      <c r="I173" s="8" t="n"/>
+      <c r="K173" s="8" t="n"/>
     </row>
     <row r="174">
       <c r="F174" s="8" t="n"/>
-      <c r="G174" s="8" t="n"/>
       <c r="H174" s="8" t="n"/>
+      <c r="I174" s="8" t="n"/>
+      <c r="K174" s="8" t="n"/>
     </row>
     <row r="175">
       <c r="F175" s="8" t="n"/>
-      <c r="G175" s="8" t="n"/>
       <c r="H175" s="8" t="n"/>
+      <c r="I175" s="8" t="n"/>
+      <c r="K175" s="8" t="n"/>
     </row>
     <row r="176">
       <c r="F176" s="8" t="n"/>
-      <c r="G176" s="8" t="n"/>
       <c r="H176" s="8" t="n"/>
+      <c r="I176" s="8" t="n"/>
+      <c r="K176" s="8" t="n"/>
     </row>
     <row r="177">
       <c r="F177" s="8" t="n"/>
-      <c r="G177" s="8" t="n"/>
       <c r="H177" s="8" t="n"/>
+      <c r="I177" s="8" t="n"/>
+      <c r="K177" s="8" t="n"/>
     </row>
     <row r="178">
       <c r="F178" s="8" t="n"/>
-      <c r="G178" s="8" t="n"/>
       <c r="H178" s="8" t="n"/>
+      <c r="I178" s="8" t="n"/>
+      <c r="K178" s="8" t="n"/>
     </row>
     <row r="179">
       <c r="F179" s="8" t="n"/>
-      <c r="G179" s="8" t="n"/>
       <c r="H179" s="8" t="n"/>
+      <c r="I179" s="8" t="n"/>
+      <c r="K179" s="8" t="n"/>
     </row>
     <row r="180">
       <c r="F180" s="8" t="n"/>
-      <c r="G180" s="8" t="n"/>
       <c r="H180" s="8" t="n"/>
+      <c r="I180" s="8" t="n"/>
+      <c r="K180" s="8" t="n"/>
     </row>
     <row r="181">
       <c r="F181" s="8" t="n"/>
-      <c r="G181" s="8" t="n"/>
       <c r="H181" s="8" t="n"/>
+      <c r="I181" s="8" t="n"/>
+      <c r="K181" s="8" t="n"/>
     </row>
     <row r="182">
       <c r="F182" s="8" t="n"/>
-      <c r="G182" s="8" t="n"/>
       <c r="H182" s="8" t="n"/>
+      <c r="I182" s="8" t="n"/>
+      <c r="K182" s="8" t="n"/>
     </row>
     <row r="183">
       <c r="F183" s="8" t="n"/>
-      <c r="G183" s="8" t="n"/>
       <c r="H183" s="8" t="n"/>
+      <c r="I183" s="8" t="n"/>
+      <c r="K183" s="8" t="n"/>
     </row>
     <row r="184">
       <c r="F184" s="8" t="n"/>
-      <c r="G184" s="8" t="n"/>
       <c r="H184" s="8" t="n"/>
+      <c r="I184" s="8" t="n"/>
+      <c r="K184" s="8" t="n"/>
     </row>
     <row r="185">
       <c r="F185" s="8" t="n"/>
-      <c r="G185" s="8" t="n"/>
       <c r="H185" s="8" t="n"/>
+      <c r="I185" s="8" t="n"/>
+      <c r="K185" s="8" t="n"/>
     </row>
     <row r="186">
       <c r="F186" s="8" t="n"/>
-      <c r="G186" s="8" t="n"/>
       <c r="H186" s="8" t="n"/>
+      <c r="I186" s="8" t="n"/>
+      <c r="K186" s="8" t="n"/>
     </row>
     <row r="187">
       <c r="F187" s="8" t="n"/>
-      <c r="G187" s="8" t="n"/>
       <c r="H187" s="8" t="n"/>
+      <c r="I187" s="8" t="n"/>
+      <c r="K187" s="8" t="n"/>
     </row>
     <row r="188">
       <c r="F188" s="8" t="n"/>
-      <c r="G188" s="8" t="n"/>
       <c r="H188" s="8" t="n"/>
+      <c r="I188" s="8" t="n"/>
+      <c r="K188" s="8" t="n"/>
     </row>
     <row r="189">
       <c r="F189" s="8" t="n"/>
-      <c r="G189" s="8" t="n"/>
       <c r="H189" s="8" t="n"/>
+      <c r="I189" s="8" t="n"/>
+      <c r="K189" s="8" t="n"/>
     </row>
     <row r="190">
       <c r="F190" s="8" t="n"/>
-      <c r="G190" s="8" t="n"/>
       <c r="H190" s="8" t="n"/>
+      <c r="I190" s="8" t="n"/>
+      <c r="K190" s="8" t="n"/>
     </row>
     <row r="191">
       <c r="F191" s="8" t="n"/>
-      <c r="G191" s="8" t="n"/>
       <c r="H191" s="8" t="n"/>
+      <c r="I191" s="8" t="n"/>
+      <c r="K191" s="8" t="n"/>
     </row>
     <row r="192">
       <c r="F192" s="8" t="n"/>
-      <c r="G192" s="8" t="n"/>
       <c r="H192" s="8" t="n"/>
+      <c r="I192" s="8" t="n"/>
+      <c r="K192" s="8" t="n"/>
     </row>
     <row r="193">
       <c r="F193" s="8" t="n"/>
-      <c r="G193" s="8" t="n"/>
       <c r="H193" s="8" t="n"/>
+      <c r="I193" s="8" t="n"/>
+      <c r="K193" s="8" t="n"/>
     </row>
     <row r="194">
       <c r="F194" s="8" t="n"/>
-      <c r="G194" s="8" t="n"/>
       <c r="H194" s="8" t="n"/>
+      <c r="I194" s="8" t="n"/>
+      <c r="K194" s="8" t="n"/>
     </row>
     <row r="195">
       <c r="F195" s="8" t="n"/>
-      <c r="G195" s="8" t="n"/>
       <c r="H195" s="8" t="n"/>
+      <c r="I195" s="8" t="n"/>
+      <c r="K195" s="8" t="n"/>
     </row>
     <row r="196">
       <c r="F196" s="8" t="n"/>
-      <c r="G196" s="8" t="n"/>
       <c r="H196" s="8" t="n"/>
+      <c r="I196" s="8" t="n"/>
+      <c r="K196" s="8" t="n"/>
     </row>
     <row r="197">
       <c r="F197" s="8" t="n"/>
-      <c r="G197" s="8" t="n"/>
       <c r="H197" s="8" t="n"/>
+      <c r="I197" s="8" t="n"/>
+      <c r="K197" s="8" t="n"/>
     </row>
     <row r="198">
       <c r="F198" s="8" t="n"/>
-      <c r="G198" s="8" t="n"/>
       <c r="H198" s="8" t="n"/>
+      <c r="I198" s="8" t="n"/>
+      <c r="K198" s="8" t="n"/>
     </row>
     <row r="199">
       <c r="F199" s="8" t="n"/>
-      <c r="G199" s="8" t="n"/>
       <c r="H199" s="8" t="n"/>
+      <c r="I199" s="8" t="n"/>
+      <c r="K199" s="8" t="n"/>
     </row>
     <row r="200">
       <c r="F200" s="8" t="n"/>
-      <c r="G200" s="8" t="n"/>
       <c r="H200" s="8" t="n"/>
+      <c r="I200" s="8" t="n"/>
+      <c r="K200" s="8" t="n"/>
     </row>
     <row r="201">
       <c r="F201" s="8" t="n"/>
-      <c r="G201" s="8" t="n"/>
       <c r="H201" s="8" t="n"/>
+      <c r="I201" s="8" t="n"/>
+      <c r="K201" s="8" t="n"/>
     </row>
     <row r="202">
       <c r="F202" s="8" t="n"/>
-      <c r="G202" s="8" t="n"/>
       <c r="H202" s="8" t="n"/>
+      <c r="I202" s="8" t="n"/>
+      <c r="K202" s="8" t="n"/>
     </row>
     <row r="203">
       <c r="F203" s="8" t="n"/>
-      <c r="G203" s="8" t="n"/>
       <c r="H203" s="8" t="n"/>
+      <c r="I203" s="8" t="n"/>
+      <c r="K203" s="8" t="n"/>
     </row>
     <row r="204">
       <c r="F204" s="8" t="n"/>
-      <c r="G204" s="8" t="n"/>
       <c r="H204" s="8" t="n"/>
+      <c r="I204" s="8" t="n"/>
+      <c r="K204" s="8" t="n"/>
     </row>
     <row r="205">
       <c r="F205" s="8" t="n"/>
-      <c r="G205" s="8" t="n"/>
       <c r="H205" s="8" t="n"/>
+      <c r="I205" s="8" t="n"/>
+      <c r="K205" s="8" t="n"/>
     </row>
     <row r="206">
       <c r="F206" s="8" t="n"/>
-      <c r="G206" s="8" t="n"/>
       <c r="H206" s="8" t="n"/>
+      <c r="I206" s="8" t="n"/>
+      <c r="K206" s="8" t="n"/>
     </row>
     <row r="207">
       <c r="F207" s="8" t="n"/>
-      <c r="G207" s="8" t="n"/>
       <c r="H207" s="8" t="n"/>
+      <c r="I207" s="8" t="n"/>
+      <c r="K207" s="8" t="n"/>
     </row>
     <row r="208">
       <c r="F208" s="8" t="n"/>
-      <c r="G208" s="8" t="n"/>
       <c r="H208" s="8" t="n"/>
+      <c r="I208" s="8" t="n"/>
+      <c r="K208" s="8" t="n"/>
     </row>
     <row r="209">
       <c r="F209" s="8" t="n"/>
-      <c r="G209" s="8" t="n"/>
       <c r="H209" s="8" t="n"/>
+      <c r="I209" s="8" t="n"/>
+      <c r="K209" s="8" t="n"/>
     </row>
     <row r="210">
       <c r="F210" s="8" t="n"/>
-      <c r="G210" s="8" t="n"/>
       <c r="H210" s="8" t="n"/>
+      <c r="I210" s="8" t="n"/>
+      <c r="K210" s="8" t="n"/>
     </row>
     <row r="211">
       <c r="F211" s="8" t="n"/>
-      <c r="G211" s="8" t="n"/>
       <c r="H211" s="8" t="n"/>
+      <c r="I211" s="8" t="n"/>
+      <c r="K211" s="8" t="n"/>
     </row>
     <row r="212">
       <c r="F212" s="8" t="n"/>
-      <c r="G212" s="8" t="n"/>
       <c r="H212" s="8" t="n"/>
+      <c r="I212" s="8" t="n"/>
+      <c r="K212" s="8" t="n"/>
     </row>
     <row r="213">
       <c r="F213" s="8" t="n"/>
-      <c r="G213" s="8" t="n"/>
       <c r="H213" s="8" t="n"/>
+      <c r="I213" s="8" t="n"/>
+      <c r="K213" s="8" t="n"/>
     </row>
     <row r="214">
       <c r="F214" s="8" t="n"/>
-      <c r="G214" s="8" t="n"/>
       <c r="H214" s="8" t="n"/>
+      <c r="I214" s="8" t="n"/>
+      <c r="K214" s="8" t="n"/>
     </row>
     <row r="215">
       <c r="F215" s="8" t="n"/>
-      <c r="G215" s="8" t="n"/>
       <c r="H215" s="8" t="n"/>
+      <c r="I215" s="8" t="n"/>
+      <c r="K215" s="8" t="n"/>
     </row>
     <row r="216">
       <c r="F216" s="8" t="n"/>
-      <c r="G216" s="8" t="n"/>
       <c r="H216" s="8" t="n"/>
+      <c r="I216" s="8" t="n"/>
+      <c r="K216" s="8" t="n"/>
     </row>
     <row r="217">
       <c r="F217" s="8" t="n"/>
-      <c r="G217" s="8" t="n"/>
       <c r="H217" s="8" t="n"/>
+      <c r="I217" s="8" t="n"/>
+      <c r="K217" s="8" t="n"/>
     </row>
     <row r="218">
       <c r="F218" s="8" t="n"/>
-      <c r="G218" s="8" t="n"/>
       <c r="H218" s="8" t="n"/>
+      <c r="I218" s="8" t="n"/>
+      <c r="K218" s="8" t="n"/>
     </row>
     <row r="219">
       <c r="F219" s="8" t="n"/>
-      <c r="G219" s="8" t="n"/>
       <c r="H219" s="8" t="n"/>
+      <c r="I219" s="8" t="n"/>
+      <c r="K219" s="8" t="n"/>
     </row>
     <row r="220">
       <c r="F220" s="8" t="n"/>
-      <c r="G220" s="8" t="n"/>
       <c r="H220" s="8" t="n"/>
+      <c r="I220" s="8" t="n"/>
+      <c r="K220" s="8" t="n"/>
     </row>
     <row r="221">
       <c r="F221" s="8" t="n"/>
-      <c r="G221" s="8" t="n"/>
       <c r="H221" s="8" t="n"/>
+      <c r="I221" s="8" t="n"/>
+      <c r="K221" s="8" t="n"/>
     </row>
     <row r="222">
       <c r="F222" s="8" t="n"/>
-      <c r="G222" s="8" t="n"/>
       <c r="H222" s="8" t="n"/>
+      <c r="I222" s="8" t="n"/>
+      <c r="K222" s="8" t="n"/>
     </row>
     <row r="223">
       <c r="F223" s="8" t="n"/>
-      <c r="G223" s="8" t="n"/>
       <c r="H223" s="8" t="n"/>
+      <c r="I223" s="8" t="n"/>
+      <c r="K223" s="8" t="n"/>
     </row>
     <row r="224">
       <c r="F224" s="8" t="n"/>
-      <c r="G224" s="8" t="n"/>
       <c r="H224" s="8" t="n"/>
+      <c r="I224" s="8" t="n"/>
+      <c r="K224" s="8" t="n"/>
     </row>
     <row r="225">
       <c r="F225" s="8" t="n"/>
-      <c r="G225" s="8" t="n"/>
       <c r="H225" s="8" t="n"/>
+      <c r="I225" s="8" t="n"/>
+      <c r="K225" s="8" t="n"/>
     </row>
     <row r="226">
       <c r="F226" s="8" t="n"/>
-      <c r="G226" s="8" t="n"/>
       <c r="H226" s="8" t="n"/>
+      <c r="I226" s="8" t="n"/>
+      <c r="K226" s="8" t="n"/>
     </row>
     <row r="227">
       <c r="F227" s="8" t="n"/>
-      <c r="G227" s="8" t="n"/>
       <c r="H227" s="8" t="n"/>
+      <c r="I227" s="8" t="n"/>
+      <c r="K227" s="8" t="n"/>
     </row>
     <row r="228">
       <c r="F228" s="8" t="n"/>
-      <c r="G228" s="8" t="n"/>
       <c r="H228" s="8" t="n"/>
+      <c r="I228" s="8" t="n"/>
+      <c r="K228" s="8" t="n"/>
     </row>
     <row r="229">
       <c r="F229" s="8" t="n"/>
-      <c r="G229" s="8" t="n"/>
       <c r="H229" s="8" t="n"/>
+      <c r="I229" s="8" t="n"/>
+      <c r="K229" s="8" t="n"/>
     </row>
     <row r="230">
       <c r="F230" s="8" t="n"/>
-      <c r="G230" s="8" t="n"/>
       <c r="H230" s="8" t="n"/>
+      <c r="I230" s="8" t="n"/>
+      <c r="K230" s="8" t="n"/>
     </row>
     <row r="231">
       <c r="F231" s="8" t="n"/>
-      <c r="G231" s="8" t="n"/>
       <c r="H231" s="8" t="n"/>
+      <c r="I231" s="8" t="n"/>
+      <c r="K231" s="8" t="n"/>
     </row>
     <row r="232">
       <c r="F232" s="8" t="n"/>
-      <c r="G232" s="8" t="n"/>
       <c r="H232" s="8" t="n"/>
+      <c r="I232" s="8" t="n"/>
+      <c r="K232" s="8" t="n"/>
     </row>
     <row r="233">
       <c r="F233" s="8" t="n"/>
-      <c r="G233" s="8" t="n"/>
       <c r="H233" s="8" t="n"/>
+      <c r="I233" s="8" t="n"/>
+      <c r="K233" s="8" t="n"/>
     </row>
     <row r="234">
       <c r="F234" s="8" t="n"/>
-      <c r="G234" s="8" t="n"/>
       <c r="H234" s="8" t="n"/>
+      <c r="I234" s="8" t="n"/>
+      <c r="K234" s="8" t="n"/>
     </row>
     <row r="235">
       <c r="F235" s="8" t="n"/>
-      <c r="G235" s="8" t="n"/>
       <c r="H235" s="8" t="n"/>
+      <c r="I235" s="8" t="n"/>
+      <c r="K235" s="8" t="n"/>
     </row>
     <row r="236">
       <c r="F236" s="8" t="n"/>
-      <c r="G236" s="8" t="n"/>
       <c r="H236" s="8" t="n"/>
+      <c r="I236" s="8" t="n"/>
+      <c r="K236" s="8" t="n"/>
     </row>
     <row r="237">
       <c r="F237" s="8" t="n"/>
-      <c r="G237" s="8" t="n"/>
       <c r="H237" s="8" t="n"/>
+      <c r="I237" s="8" t="n"/>
+      <c r="K237" s="8" t="n"/>
     </row>
     <row r="238">
       <c r="F238" s="8" t="n"/>
-      <c r="G238" s="8" t="n"/>
       <c r="H238" s="8" t="n"/>
+      <c r="I238" s="8" t="n"/>
+      <c r="K238" s="8" t="n"/>
     </row>
     <row r="239">
       <c r="F239" s="8" t="n"/>
-      <c r="G239" s="8" t="n"/>
       <c r="H239" s="8" t="n"/>
+      <c r="I239" s="8" t="n"/>
+      <c r="K239" s="8" t="n"/>
     </row>
     <row r="240">
       <c r="F240" s="8" t="n"/>
-      <c r="G240" s="8" t="n"/>
       <c r="H240" s="8" t="n"/>
+      <c r="I240" s="8" t="n"/>
+      <c r="K240" s="8" t="n"/>
     </row>
     <row r="241">
       <c r="F241" s="8" t="n"/>
-      <c r="G241" s="8" t="n"/>
       <c r="H241" s="8" t="n"/>
+      <c r="I241" s="8" t="n"/>
+      <c r="K241" s="8" t="n"/>
     </row>
     <row r="242">
       <c r="F242" s="8" t="n"/>
-      <c r="G242" s="8" t="n"/>
       <c r="H242" s="8" t="n"/>
+      <c r="I242" s="8" t="n"/>
+      <c r="K242" s="8" t="n"/>
     </row>
     <row r="243">
       <c r="F243" s="8" t="n"/>
-      <c r="G243" s="8" t="n"/>
       <c r="H243" s="8" t="n"/>
+      <c r="I243" s="8" t="n"/>
+      <c r="K243" s="8" t="n"/>
     </row>
     <row r="244">
       <c r="F244" s="8" t="n"/>
-      <c r="G244" s="8" t="n"/>
       <c r="H244" s="8" t="n"/>
+      <c r="I244" s="8" t="n"/>
+      <c r="K244" s="8" t="n"/>
     </row>
     <row r="245">
       <c r="F245" s="8" t="n"/>
-      <c r="G245" s="8" t="n"/>
       <c r="H245" s="8" t="n"/>
+      <c r="I245" s="8" t="n"/>
+      <c r="K245" s="8" t="n"/>
     </row>
     <row r="246">
       <c r="F246" s="8" t="n"/>
-      <c r="G246" s="8" t="n"/>
       <c r="H246" s="8" t="n"/>
+      <c r="I246" s="8" t="n"/>
+      <c r="K246" s="8" t="n"/>
     </row>
     <row r="247">
       <c r="F247" s="8" t="n"/>
-      <c r="G247" s="8" t="n"/>
       <c r="H247" s="8" t="n"/>
+      <c r="I247" s="8" t="n"/>
+      <c r="K247" s="8" t="n"/>
     </row>
     <row r="248">
       <c r="F248" s="8" t="n"/>
-      <c r="G248" s="8" t="n"/>
       <c r="H248" s="8" t="n"/>
+      <c r="I248" s="8" t="n"/>
+      <c r="K248" s="8" t="n"/>
     </row>
     <row r="249">
       <c r="F249" s="8" t="n"/>
-      <c r="G249" s="8" t="n"/>
       <c r="H249" s="8" t="n"/>
+      <c r="I249" s="8" t="n"/>
+      <c r="K249" s="8" t="n"/>
     </row>
     <row r="250">
       <c r="F250" s="8" t="n"/>
-      <c r="G250" s="8" t="n"/>
       <c r="H250" s="8" t="n"/>
+      <c r="I250" s="8" t="n"/>
+      <c r="K250" s="8" t="n"/>
     </row>
     <row r="251">
       <c r="F251" s="8" t="n"/>
-      <c r="G251" s="8" t="n"/>
       <c r="H251" s="8" t="n"/>
+      <c r="I251" s="8" t="n"/>
+      <c r="K251" s="8" t="n"/>
     </row>
     <row r="252">
       <c r="F252" s="8" t="n"/>
-      <c r="G252" s="8" t="n"/>
       <c r="H252" s="8" t="n"/>
+      <c r="I252" s="8" t="n"/>
+      <c r="K252" s="8" t="n"/>
     </row>
     <row r="253">
       <c r="F253" s="8" t="n"/>
-      <c r="G253" s="8" t="n"/>
       <c r="H253" s="8" t="n"/>
+      <c r="I253" s="8" t="n"/>
+      <c r="K253" s="8" t="n"/>
     </row>
     <row r="254">
       <c r="F254" s="8" t="n"/>
-      <c r="G254" s="8" t="n"/>
       <c r="H254" s="8" t="n"/>
+      <c r="I254" s="8" t="n"/>
+      <c r="K254" s="8" t="n"/>
     </row>
     <row r="255">
       <c r="F255" s="8" t="n"/>
-      <c r="G255" s="8" t="n"/>
       <c r="H255" s="8" t="n"/>
+      <c r="I255" s="8" t="n"/>
+      <c r="K255" s="8" t="n"/>
     </row>
     <row r="256">
       <c r="F256" s="8" t="n"/>
-      <c r="G256" s="8" t="n"/>
       <c r="H256" s="8" t="n"/>
+      <c r="I256" s="8" t="n"/>
+      <c r="K256" s="8" t="n"/>
     </row>
     <row r="257">
       <c r="F257" s="8" t="n"/>
-      <c r="G257" s="8" t="n"/>
       <c r="H257" s="8" t="n"/>
+      <c r="I257" s="8" t="n"/>
+      <c r="K257" s="8" t="n"/>
     </row>
     <row r="258">
       <c r="F258" s="8" t="n"/>
-      <c r="G258" s="8" t="n"/>
       <c r="H258" s="8" t="n"/>
+      <c r="I258" s="8" t="n"/>
+      <c r="K258" s="8" t="n"/>
     </row>
     <row r="259">
       <c r="F259" s="8" t="n"/>
-      <c r="G259" s="8" t="n"/>
       <c r="H259" s="8" t="n"/>
+      <c r="I259" s="8" t="n"/>
+      <c r="K259" s="8" t="n"/>
     </row>
     <row r="260">
       <c r="F260" s="8" t="n"/>
-      <c r="G260" s="8" t="n"/>
       <c r="H260" s="8" t="n"/>
+      <c r="I260" s="8" t="n"/>
+      <c r="K260" s="8" t="n"/>
     </row>
     <row r="261">
       <c r="F261" s="8" t="n"/>
-      <c r="G261" s="8" t="n"/>
       <c r="H261" s="8" t="n"/>
+      <c r="I261" s="8" t="n"/>
+      <c r="K261" s="8" t="n"/>
     </row>
     <row r="262">
       <c r="F262" s="8" t="n"/>
-      <c r="G262" s="8" t="n"/>
       <c r="H262" s="8" t="n"/>
+      <c r="I262" s="8" t="n"/>
+      <c r="K262" s="8" t="n"/>
     </row>
     <row r="263">
       <c r="F263" s="8" t="n"/>
-      <c r="G263" s="8" t="n"/>
       <c r="H263" s="8" t="n"/>
+      <c r="I263" s="8" t="n"/>
+      <c r="K263" s="8" t="n"/>
     </row>
     <row r="264">
       <c r="F264" s="8" t="n"/>
-      <c r="G264" s="8" t="n"/>
       <c r="H264" s="8" t="n"/>
+      <c r="I264" s="8" t="n"/>
+      <c r="K264" s="8" t="n"/>
     </row>
     <row r="265">
       <c r="F265" s="8" t="n"/>
-      <c r="G265" s="8" t="n"/>
       <c r="H265" s="8" t="n"/>
+      <c r="I265" s="8" t="n"/>
+      <c r="K265" s="8" t="n"/>
     </row>
     <row r="266">
       <c r="F266" s="8" t="n"/>
-      <c r="G266" s="8" t="n"/>
       <c r="H266" s="8" t="n"/>
+      <c r="I266" s="8" t="n"/>
+      <c r="K266" s="8" t="n"/>
     </row>
     <row r="267">
       <c r="F267" s="8" t="n"/>
-      <c r="G267" s="8" t="n"/>
       <c r="H267" s="8" t="n"/>
+      <c r="I267" s="8" t="n"/>
+      <c r="K267" s="8" t="n"/>
     </row>
     <row r="268">
       <c r="F268" s="8" t="n"/>
-      <c r="G268" s="8" t="n"/>
       <c r="H268" s="8" t="n"/>
+      <c r="I268" s="8" t="n"/>
+      <c r="K268" s="8" t="n"/>
     </row>
     <row r="269">
       <c r="F269" s="8" t="n"/>
-      <c r="G269" s="8" t="n"/>
       <c r="H269" s="8" t="n"/>
+      <c r="I269" s="8" t="n"/>
+      <c r="K269" s="8" t="n"/>
     </row>
     <row r="270">
       <c r="F270" s="8" t="n"/>
-      <c r="G270" s="8" t="n"/>
       <c r="H270" s="8" t="n"/>
+      <c r="I270" s="8" t="n"/>
+      <c r="K270" s="8" t="n"/>
     </row>
     <row r="271">
       <c r="F271" s="8" t="n"/>
-      <c r="G271" s="8" t="n"/>
       <c r="H271" s="8" t="n"/>
+      <c r="I271" s="8" t="n"/>
+      <c r="K271" s="8" t="n"/>
     </row>
     <row r="272">
       <c r="F272" s="8" t="n"/>
-      <c r="G272" s="8" t="n"/>
       <c r="H272" s="8" t="n"/>
+      <c r="I272" s="8" t="n"/>
+      <c r="K272" s="8" t="n"/>
     </row>
     <row r="273">
       <c r="F273" s="8" t="n"/>
-      <c r="G273" s="8" t="n"/>
       <c r="H273" s="8" t="n"/>
+      <c r="I273" s="8" t="n"/>
+      <c r="K273" s="8" t="n"/>
     </row>
     <row r="274">
       <c r="F274" s="8" t="n"/>
-      <c r="G274" s="8" t="n"/>
       <c r="H274" s="8" t="n"/>
+      <c r="I274" s="8" t="n"/>
+      <c r="K274" s="8" t="n"/>
     </row>
     <row r="275">
       <c r="F275" s="8" t="n"/>
-      <c r="G275" s="8" t="n"/>
       <c r="H275" s="8" t="n"/>
+      <c r="I275" s="8" t="n"/>
+      <c r="K275" s="8" t="n"/>
     </row>
     <row r="276">
       <c r="F276" s="8" t="n"/>
-      <c r="G276" s="8" t="n"/>
       <c r="H276" s="8" t="n"/>
+      <c r="I276" s="8" t="n"/>
+      <c r="K276" s="8" t="n"/>
     </row>
     <row r="277">
       <c r="F277" s="8" t="n"/>
-      <c r="G277" s="8" t="n"/>
       <c r="H277" s="8" t="n"/>
+      <c r="I277" s="8" t="n"/>
+      <c r="K277" s="8" t="n"/>
     </row>
     <row r="278">
       <c r="F278" s="8" t="n"/>
-      <c r="G278" s="8" t="n"/>
       <c r="H278" s="8" t="n"/>
+      <c r="I278" s="8" t="n"/>
+      <c r="K278" s="8" t="n"/>
     </row>
     <row r="279">
       <c r="F279" s="8" t="n"/>
-      <c r="G279" s="8" t="n"/>
       <c r="H279" s="8" t="n"/>
+      <c r="I279" s="8" t="n"/>
+      <c r="K279" s="8" t="n"/>
     </row>
     <row r="280">
       <c r="F280" s="8" t="n"/>
-      <c r="G280" s="8" t="n"/>
       <c r="H280" s="8" t="n"/>
+      <c r="I280" s="8" t="n"/>
+      <c r="K280" s="8" t="n"/>
     </row>
     <row r="281">
       <c r="F281" s="8" t="n"/>
-      <c r="G281" s="8" t="n"/>
       <c r="H281" s="8" t="n"/>
+      <c r="I281" s="8" t="n"/>
+      <c r="K281" s="8" t="n"/>
     </row>
     <row r="282">
       <c r="F282" s="8" t="n"/>
-      <c r="G282" s="8" t="n"/>
       <c r="H282" s="8" t="n"/>
+      <c r="I282" s="8" t="n"/>
+      <c r="K282" s="8" t="n"/>
     </row>
     <row r="283">
       <c r="F283" s="8" t="n"/>
-      <c r="G283" s="8" t="n"/>
       <c r="H283" s="8" t="n"/>
+      <c r="I283" s="8" t="n"/>
+      <c r="K283" s="8" t="n"/>
     </row>
     <row r="284">
       <c r="F284" s="8" t="n"/>
-      <c r="G284" s="8" t="n"/>
       <c r="H284" s="8" t="n"/>
+      <c r="I284" s="8" t="n"/>
+      <c r="K284" s="8" t="n"/>
     </row>
     <row r="285">
       <c r="F285" s="8" t="n"/>
-      <c r="G285" s="8" t="n"/>
       <c r="H285" s="8" t="n"/>
+      <c r="I285" s="8" t="n"/>
+      <c r="K285" s="8" t="n"/>
     </row>
     <row r="286">
       <c r="F286" s="8" t="n"/>
-      <c r="G286" s="8" t="n"/>
       <c r="H286" s="8" t="n"/>
+      <c r="I286" s="8" t="n"/>
+      <c r="K286" s="8" t="n"/>
     </row>
     <row r="287">
       <c r="F287" s="8" t="n"/>
-      <c r="G287" s="8" t="n"/>
       <c r="H287" s="8" t="n"/>
+      <c r="I287" s="8" t="n"/>
+      <c r="K287" s="8" t="n"/>
     </row>
     <row r="288">
       <c r="F288" s="8" t="n"/>
-      <c r="G288" s="8" t="n"/>
       <c r="H288" s="8" t="n"/>
+      <c r="I288" s="8" t="n"/>
+      <c r="K288" s="8" t="n"/>
     </row>
     <row r="289">
       <c r="F289" s="8" t="n"/>
-      <c r="G289" s="8" t="n"/>
       <c r="H289" s="8" t="n"/>
+      <c r="I289" s="8" t="n"/>
+      <c r="K289" s="8" t="n"/>
     </row>
     <row r="290">
       <c r="F290" s="8" t="n"/>
-      <c r="G290" s="8" t="n"/>
       <c r="H290" s="8" t="n"/>
+      <c r="I290" s="8" t="n"/>
+      <c r="K290" s="8" t="n"/>
     </row>
     <row r="291">
       <c r="F291" s="8" t="n"/>
-      <c r="G291" s="8" t="n"/>
       <c r="H291" s="8" t="n"/>
+      <c r="I291" s="8" t="n"/>
+      <c r="K291" s="8" t="n"/>
     </row>
     <row r="292">
       <c r="F292" s="8" t="n"/>
-      <c r="G292" s="8" t="n"/>
       <c r="H292" s="8" t="n"/>
+      <c r="I292" s="8" t="n"/>
+      <c r="K292" s="8" t="n"/>
     </row>
     <row r="293">
       <c r="F293" s="8" t="n"/>
-      <c r="G293" s="8" t="n"/>
       <c r="H293" s="8" t="n"/>
+      <c r="I293" s="8" t="n"/>
+      <c r="K293" s="8" t="n"/>
     </row>
     <row r="294">
       <c r="F294" s="8" t="n"/>
-      <c r="G294" s="8" t="n"/>
       <c r="H294" s="8" t="n"/>
+      <c r="I294" s="8" t="n"/>
+      <c r="K294" s="8" t="n"/>
     </row>
     <row r="295">
       <c r="F295" s="8" t="n"/>
-      <c r="G295" s="8" t="n"/>
       <c r="H295" s="8" t="n"/>
+      <c r="I295" s="8" t="n"/>
+      <c r="K295" s="8" t="n"/>
     </row>
     <row r="296">
       <c r="F296" s="8" t="n"/>
-      <c r="G296" s="8" t="n"/>
       <c r="H296" s="8" t="n"/>
+      <c r="I296" s="8" t="n"/>
+      <c r="K296" s="8" t="n"/>
     </row>
     <row r="297">
       <c r="F297" s="8" t="n"/>
-      <c r="G297" s="8" t="n"/>
       <c r="H297" s="8" t="n"/>
+      <c r="I297" s="8" t="n"/>
+      <c r="K297" s="8" t="n"/>
     </row>
     <row r="298">
       <c r="F298" s="8" t="n"/>
-      <c r="G298" s="8" t="n"/>
       <c r="H298" s="8" t="n"/>
+      <c r="I298" s="8" t="n"/>
+      <c r="K298" s="8" t="n"/>
     </row>
     <row r="299">
       <c r="F299" s="8" t="n"/>
-      <c r="G299" s="8" t="n"/>
       <c r="H299" s="8" t="n"/>
+      <c r="I299" s="8" t="n"/>
+      <c r="K299" s="8" t="n"/>
     </row>
     <row r="300">
       <c r="F300" s="8" t="n"/>
-      <c r="G300" s="8" t="n"/>
       <c r="H300" s="8" t="n"/>
+      <c r="I300" s="8" t="n"/>
+      <c r="K300" s="8" t="n"/>
     </row>
     <row r="301">
       <c r="F301" s="8" t="n"/>
-      <c r="G301" s="8" t="n"/>
       <c r="H301" s="8" t="n"/>
+      <c r="I301" s="8" t="n"/>
+      <c r="K301" s="8" t="n"/>
     </row>
     <row r="302">
       <c r="F302" s="8" t="n"/>
-      <c r="G302" s="8" t="n"/>
       <c r="H302" s="8" t="n"/>
+      <c r="I302" s="8" t="n"/>
+      <c r="K302" s="8" t="n"/>
     </row>
     <row r="303">
       <c r="F303" s="8" t="n"/>
-      <c r="G303" s="8" t="n"/>
       <c r="H303" s="8" t="n"/>
+      <c r="I303" s="8" t="n"/>
+      <c r="K303" s="8" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation sqref="C4:C303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Integer" error="请填非负整数。" type="whole" errorStyle="warning" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="I4:I303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
+    <dataValidation sqref="G4:G303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
+      <formula1>Lists!$AE$2:$AE$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="L4:L303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
+      <formula1>Lists!$AF$2:$AF$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="N4:N303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
       <formula1>Lists!$AD$2:$AD$4</formula1>
     </dataValidation>
-    <dataValidation sqref="K4:K303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
+    <dataValidation sqref="P4:P303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
       <formula1>Lists!$AC$2:$AC$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Full-text logs: blank n_children_aggregate counts as 0 in compare, check warns on blank for Include; align guide and workbooks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -561,7 +561,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>数据提取工作簿（模板，草稿）v2026-10-19a — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
+          <t>数据提取工作簿（模板，草稿）v2026-10-19b — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
         </is>
       </c>
     </row>
@@ -1927,7 +1927,7 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>整数</t>
+          <t>整数；Include 时没有汇总儿童就填 0</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Drop the full-text time log (FT_time_log): scripts, workbooks, guide, protocol v1.6, manuscript draft
The change is stated as a fact only; no reason has been given by the author.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -9,14 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FT_log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FT_time_log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX_time_log" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPD_requests" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX_time_log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPD_requests" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -552,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -561,7 +560,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>数据提取工作簿（模板，草稿）v2026-10-19b — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
+          <t>数据提取工作簿（模板，草稿）v2026-10-19c — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
         </is>
       </c>
     </row>
@@ -673,1013 +672,105 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• FT_time_log：全文筛选的时间记录。每次开始和结束都写一行（日期、起止时间、处理的篇数），用来代替 Rayyan 的时间戳日志。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
+          <t>• Reports、Patients：数据提取。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• Reports、Patients：数据提取。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="36" customHeight="1">
+          <t>• EX_time_log：数据提取的时间记录，每次开始和结束都写一行（日期、起止时间、处理的报告数和录入的患者数）。这是 Claude 的建议，待确认；没有它，电子表格里看不出每份记录是怎么做出来的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>• EX_time_log：数据提取的时间记录，和 FT_time_log 一样，每次开始和结束都写一行（日期、起止时间、处理的报告数和录入的患者数）。这是 Claude 的建议，待确认；没有它，电子表格里看不出每份记录是怎么做出来的。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="54" customHeight="1">
+          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周；一报告一行）。联系记录列（2026 年 10 月 19 日加入）：第一封的送达结果、论文邮箱之外用过的途径和日期、是否联系上作者、逐次联系的日志，规则见《IPD 索取邮件》第 1、5 节。邮箱地址和退信邮件都不放进这份表。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• IPD_requests：向只有汇总数据的报告的作者索取个体数据的登记（协议第 14 节：两封邮件，间隔 4 周；一报告一行）。联系记录列（2026 年 10 月 19 日加入）：第一封的送达结果、论文邮箱之外用过的途径和日期、是否联系上作者、逐次联系的日志，规则见《IPD 索取邮件》第 1、5 节。邮箱地址和退信邮件都不放进这份表。</t>
+          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>• Rules：时间换算 9 条规则、衍生变量定义、主要暴露和结局的协议原文。</t>
+          <t>• Duration_calc：时间换算计算器。Lists：下拉列表（请勿改动，改了会影响所有表）。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• Duration_calc：时间换算计算器。Lists：下拉列表（请勿改动，改了会影响所有表）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>3. 与附录 C 的差异（Claude 的操作化，待三位确认）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
         </is>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>• A1  附录 C 的 A 部分（报告）单独放在 Reports 表，B–F 部分在 Patients 表；项目一个不少，只是不在每个患者行里重复。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="36" customHeight="1">
+          <t>• A2  '伴随疾病'多选项拆成独立的 Yes/No/NR 列；影像学检查方式拆成 US、Doppler US、CT、MRI 四列。另外加了胰尾扭转、肠梗阻两列，因为协议第 13 节的附加结局列了它们。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>• A2  '伴随疾病'多选项拆成独立的 Yes/No/NR 列；影像学检查方式拆成 US、Doppler US、CT、MRI 四列。另外加了胰尾扭转、肠梗阻两列，因为协议第 13 节的附加结局列了它们。</t>
+          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
         </is>
       </c>
     </row>
     <row r="26" ht="54" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>• A3  Procedure 在协议五项之外加了 No operation（协议第 7 节：未手术的儿童做描述性汇总）和 NR；Fixation technique 加了 Not applicable 和 NR；Approach、Viability、Basis of viability 加了 Not applicable（未手术）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="54" customHeight="1">
+          <t>• A4  加了衍生列（灰色）：own_patient（敏感性分析 1）、idx_dur_category（四类，边界见 Rules D2）、thrombocytosis（&gt;450）、primary_outcome（Rules D3）、pub_period（第 16 节的发表时期）。这些是 Claude 对协议第 12、16 节的读法，须三位确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>• A4  加了衍生列（灰色）：own_patient（敏感性分析 1）、idx_dur_category（四类，边界见 Rules D2）、thrombocytosis（&gt;450）、primary_outcome（Rules D3）、pub_period（第 16 节的发表时期）。这些是 Claude 对协议第 12、16 节的读法，须三位确认。</t>
+          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
         </is>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>• A5  ws_basis：记录报告凭什么说是游走脾（影像显示异位或活动、手术所见、只写了游走脾、只写了脾扭转而没写位置）。这是为了在全文指南 D1 的'宽松加标记'方案下，将来能做'只看有明确异位依据的'敏感分析；该敏感分析不在已注册的 8 个里，若要做须作为新增分析声明。</t>
+          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
         </is>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>• A6  加了 extractor、date_extracted、same_patient_as、idx_dur_rules、idx_dur_lower_bound、idx_dur_cat_imprecise（规则 5 和 9 要求标记）、src_* 出处列。</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
           <t>• A7  Age 的取值：协议写'年，两位小数（月数 ÷ 12）'；未报告填 NR；原文写法另存 age_verbatim。只写'child'或'患儿'而没有具体年龄的，年龄填 NR（见全文指南 D2）。</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>4. 没有验证的事</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="54" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>• 灰色列的公式用 Python 的 formulas 库按公式文本计算过（九行虚构的测试数据，覆盖各分支，没有保存）；容器里没有 Excel，也没有 LibreOffice 的 Calc，所以文件没有在 Excel 或 WPS 里打开过，下拉列表和版面实际是否正常没有验证。第一次用时请随便填几行试一下，有问题告诉 Claude。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00BBBBBB"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AF11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="36" customWidth="1" min="17" max="17"/>
-    <col width="42" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="44" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="30" customWidth="1" min="27" max="27"/>
-    <col width="40" customWidth="1" min="28" max="28"/>
-    <col width="37" customWidth="1" min="29" max="29"/>
-    <col width="14" customWidth="1" min="30" max="30"/>
-    <col width="18" customWidth="1" min="31" max="31"/>
-    <col width="14" customWidth="1" min="32" max="32"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>yn</t>
-        </is>
-      </c>
-      <c r="B1" s="17" t="inlineStr">
-        <is>
-          <t>yn_nr</t>
-        </is>
-      </c>
-      <c r="C1" s="17" t="inlineStr">
-        <is>
-          <t>sex</t>
-        </is>
-      </c>
-      <c r="D1" s="17" t="inlineStr">
-        <is>
-          <t>lang</t>
-        </is>
-      </c>
-      <c r="E1" s="17" t="inlineStr">
-        <is>
-          <t>ft_lang</t>
-        </is>
-      </c>
-      <c r="F1" s="17" t="inlineStr">
-        <is>
-          <t>design</t>
-        </is>
-      </c>
-      <c r="G1" s="17" t="inlineStr">
-        <is>
-          <t>consecutive</t>
-        </is>
-      </c>
-      <c r="H1" s="17" t="inlineStr">
-        <is>
-          <t>aetiology</t>
-        </is>
-      </c>
-      <c r="I1" s="17" t="inlineStr">
-        <is>
-          <t>ws_basis</t>
-        </is>
-      </c>
-      <c r="J1" s="17" t="inlineStr">
-        <is>
-          <t>presentation</t>
-        </is>
-      </c>
-      <c r="K1" s="17" t="inlineStr">
-        <is>
-          <t>deferred_reason</t>
-        </is>
-      </c>
-      <c r="L1" s="17" t="inlineStr">
-        <is>
-          <t>torsion_awaiting</t>
-        </is>
-      </c>
-      <c r="M1" s="17" t="inlineStr">
-        <is>
-          <t>perfusion</t>
-        </is>
-      </c>
-      <c r="N1" s="17" t="inlineStr">
-        <is>
-          <t>approach</t>
-        </is>
-      </c>
-      <c r="O1" s="17" t="inlineStr">
-        <is>
-          <t>viability</t>
-        </is>
-      </c>
-      <c r="P1" s="17" t="inlineStr">
-        <is>
-          <t>viab_basis</t>
-        </is>
-      </c>
-      <c r="Q1" s="17" t="inlineStr">
-        <is>
-          <t>procedure</t>
-        </is>
-      </c>
-      <c r="R1" s="17" t="inlineStr">
-        <is>
-          <t>fixation</t>
-        </is>
-      </c>
-      <c r="S1" s="17" t="inlineStr">
-        <is>
-          <t>reason_removed</t>
-        </is>
-      </c>
-      <c r="T1" s="17" t="inlineStr">
-        <is>
-          <t>status_fu</t>
-        </is>
-      </c>
-      <c r="U1" s="17" t="inlineStr">
-        <is>
-          <t>dur_category</t>
-        </is>
-      </c>
-      <c r="V1" s="17" t="inlineStr">
-        <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="W1" s="17" t="inlineStr">
-        <is>
-          <t>phrase</t>
-        </is>
-      </c>
-      <c r="X1" s="17" t="inlineStr">
-        <is>
-          <t>extractor</t>
-        </is>
-      </c>
-      <c r="Y1" s="17" t="inlineStr">
-        <is>
-          <t>ft_reviewer</t>
-        </is>
-      </c>
-      <c r="Z1" s="17" t="inlineStr">
-        <is>
-          <t>ft_decision</t>
-        </is>
-      </c>
-      <c r="AA1" s="17" t="inlineStr">
-        <is>
-          <t>ft_reason</t>
-        </is>
-      </c>
-      <c r="AB1" s="17" t="inlineStr">
-        <is>
-          <t>route</t>
-        </is>
-      </c>
-      <c r="AC1" s="17" t="inlineStr">
-        <is>
-          <t>ipd_final</t>
-        </is>
-      </c>
-      <c r="AD1" s="17" t="inlineStr">
-        <is>
-          <t>ipd_received</t>
-        </is>
-      </c>
-      <c r="AE1" s="17" t="inlineStr">
-        <is>
-          <t>ipd_delivery</t>
-        </is>
-      </c>
-      <c r="AF1" s="17" t="inlineStr">
-        <is>
-          <t>ipd_reached</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Case report</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Congenital</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Imaging shows ectopic position or mobility</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Acute</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Family declined</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Viable</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Intraoperative</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Detorsion only</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Mesh</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Failure of fixation</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Preserved</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>&lt;=2 d</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>hours</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>Include</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>L other language</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>Publisher or open access</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>Not yet sent</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Chinese</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Chinese</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Case series</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Acquired</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Operation shows ectopic position or mobility</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Chronic or intermittent</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Observation advised</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Reduced</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Laparoscopic</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Partially non-viable</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Histology</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Splenopexy</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Retroperitoneal or extraperitoneal pouch</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Surgeon's preference</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Partially preserved</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>3-7 d</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>days</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Less than 24 hours / a few hours / overnight</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>E2</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>Exclude</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>D no full text</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Library subscription</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>Included with IPD</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>Sent, no bounce</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Cohort</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Imaging and operation</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Acute on chronic</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Elective operation scheduled</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Converted</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Non-viable</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Partial splenectomy +/- splenopexy</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Omental wrap</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Lost</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>8-30 d</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>weeks</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Consensus</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Consensus</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>Pending IPD</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>E1 non-human</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>Interlibrary loan or document delivery</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>Narrative only (no individual data)</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Bounced</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Letter</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Named wandering spleen, no detail</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Asymptomatic</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Total splenectomy</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Direct suture</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>&gt;30 d</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>E2 not wandering spleen</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>CNKI or Wanfang</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Not eligible after check</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>No address found</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Review with new patients</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Torsion only, position not stated</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Mass only</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Autotransplantation</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Other (specify)</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>E3 adults only</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Contact author</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>No operation</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>E4 no original patient data</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>E5 not a formal article</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>Not obtained</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>E6 other</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>A aggregate data only</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>N age not confirmed under 18</t>
         </is>
       </c>
     </row>
@@ -7987,1033 +7078,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F303"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>reviewer</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>start</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>end</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>n_reports</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="62" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Reviewer</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Session start</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Session end</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Reports handled</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="100" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>yyyy-mm-dd</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>R1 = 舒俊，R2 = 卞红强（全文阶段）</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>开始时间 hh:mm（本地时间）</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>结束时间 hh:mm</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>这一段时间处理了多少篇（整数）</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>例如中断原因、遇到的疑问</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="8" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="8" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="8" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="8" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="8" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="8" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="8" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="8" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="8" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="8" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="8" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="8" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="8" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="8" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="8" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="8" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="8" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="8" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="8" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="8" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="8" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="8" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="8" t="n"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="8" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="8" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="8" t="n"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="8" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="8" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="8" t="n"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="8" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="8" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="8" t="n"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="8" t="n"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="8" t="n"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="8" t="n"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="8" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="8" t="n"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="8" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="8" t="n"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="8" t="n"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="8" t="n"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="8" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="8" t="n"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="8" t="n"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="8" t="n"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="8" t="n"/>
-    </row>
-    <row r="124">
-      <c r="A124" s="8" t="n"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="8" t="n"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="8" t="n"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="n"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="8" t="n"/>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="n"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="n"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="n"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="8" t="n"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="8" t="n"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="8" t="n"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="8" t="n"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="8" t="n"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="8" t="n"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="8" t="n"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="8" t="n"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="8" t="n"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="8" t="n"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="8" t="n"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="8" t="n"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="8" t="n"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="8" t="n"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="8" t="n"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="8" t="n"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="8" t="n"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="8" t="n"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="8" t="n"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="8" t="n"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="8" t="n"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="8" t="n"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="8" t="n"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="8" t="n"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="8" t="n"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="8" t="n"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="8" t="n"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="8" t="n"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="8" t="n"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="8" t="n"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="8" t="n"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="8" t="n"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="8" t="n"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="8" t="n"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="8" t="n"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="8" t="n"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="8" t="n"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="8" t="n"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="8" t="n"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="8" t="n"/>
-    </row>
-    <row r="172">
-      <c r="A172" s="8" t="n"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="8" t="n"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="8" t="n"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="8" t="n"/>
-    </row>
-    <row r="176">
-      <c r="A176" s="8" t="n"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="8" t="n"/>
-    </row>
-    <row r="178">
-      <c r="A178" s="8" t="n"/>
-    </row>
-    <row r="179">
-      <c r="A179" s="8" t="n"/>
-    </row>
-    <row r="180">
-      <c r="A180" s="8" t="n"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="8" t="n"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="8" t="n"/>
-    </row>
-    <row r="183">
-      <c r="A183" s="8" t="n"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="8" t="n"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="8" t="n"/>
-    </row>
-    <row r="186">
-      <c r="A186" s="8" t="n"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="8" t="n"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="8" t="n"/>
-    </row>
-    <row r="189">
-      <c r="A189" s="8" t="n"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="8" t="n"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="8" t="n"/>
-    </row>
-    <row r="192">
-      <c r="A192" s="8" t="n"/>
-    </row>
-    <row r="193">
-      <c r="A193" s="8" t="n"/>
-    </row>
-    <row r="194">
-      <c r="A194" s="8" t="n"/>
-    </row>
-    <row r="195">
-      <c r="A195" s="8" t="n"/>
-    </row>
-    <row r="196">
-      <c r="A196" s="8" t="n"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="8" t="n"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="8" t="n"/>
-    </row>
-    <row r="199">
-      <c r="A199" s="8" t="n"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="8" t="n"/>
-    </row>
-    <row r="201">
-      <c r="A201" s="8" t="n"/>
-    </row>
-    <row r="202">
-      <c r="A202" s="8" t="n"/>
-    </row>
-    <row r="203">
-      <c r="A203" s="8" t="n"/>
-    </row>
-    <row r="204">
-      <c r="A204" s="8" t="n"/>
-    </row>
-    <row r="205">
-      <c r="A205" s="8" t="n"/>
-    </row>
-    <row r="206">
-      <c r="A206" s="8" t="n"/>
-    </row>
-    <row r="207">
-      <c r="A207" s="8" t="n"/>
-    </row>
-    <row r="208">
-      <c r="A208" s="8" t="n"/>
-    </row>
-    <row r="209">
-      <c r="A209" s="8" t="n"/>
-    </row>
-    <row r="210">
-      <c r="A210" s="8" t="n"/>
-    </row>
-    <row r="211">
-      <c r="A211" s="8" t="n"/>
-    </row>
-    <row r="212">
-      <c r="A212" s="8" t="n"/>
-    </row>
-    <row r="213">
-      <c r="A213" s="8" t="n"/>
-    </row>
-    <row r="214">
-      <c r="A214" s="8" t="n"/>
-    </row>
-    <row r="215">
-      <c r="A215" s="8" t="n"/>
-    </row>
-    <row r="216">
-      <c r="A216" s="8" t="n"/>
-    </row>
-    <row r="217">
-      <c r="A217" s="8" t="n"/>
-    </row>
-    <row r="218">
-      <c r="A218" s="8" t="n"/>
-    </row>
-    <row r="219">
-      <c r="A219" s="8" t="n"/>
-    </row>
-    <row r="220">
-      <c r="A220" s="8" t="n"/>
-    </row>
-    <row r="221">
-      <c r="A221" s="8" t="n"/>
-    </row>
-    <row r="222">
-      <c r="A222" s="8" t="n"/>
-    </row>
-    <row r="223">
-      <c r="A223" s="8" t="n"/>
-    </row>
-    <row r="224">
-      <c r="A224" s="8" t="n"/>
-    </row>
-    <row r="225">
-      <c r="A225" s="8" t="n"/>
-    </row>
-    <row r="226">
-      <c r="A226" s="8" t="n"/>
-    </row>
-    <row r="227">
-      <c r="A227" s="8" t="n"/>
-    </row>
-    <row r="228">
-      <c r="A228" s="8" t="n"/>
-    </row>
-    <row r="229">
-      <c r="A229" s="8" t="n"/>
-    </row>
-    <row r="230">
-      <c r="A230" s="8" t="n"/>
-    </row>
-    <row r="231">
-      <c r="A231" s="8" t="n"/>
-    </row>
-    <row r="232">
-      <c r="A232" s="8" t="n"/>
-    </row>
-    <row r="233">
-      <c r="A233" s="8" t="n"/>
-    </row>
-    <row r="234">
-      <c r="A234" s="8" t="n"/>
-    </row>
-    <row r="235">
-      <c r="A235" s="8" t="n"/>
-    </row>
-    <row r="236">
-      <c r="A236" s="8" t="n"/>
-    </row>
-    <row r="237">
-      <c r="A237" s="8" t="n"/>
-    </row>
-    <row r="238">
-      <c r="A238" s="8" t="n"/>
-    </row>
-    <row r="239">
-      <c r="A239" s="8" t="n"/>
-    </row>
-    <row r="240">
-      <c r="A240" s="8" t="n"/>
-    </row>
-    <row r="241">
-      <c r="A241" s="8" t="n"/>
-    </row>
-    <row r="242">
-      <c r="A242" s="8" t="n"/>
-    </row>
-    <row r="243">
-      <c r="A243" s="8" t="n"/>
-    </row>
-    <row r="244">
-      <c r="A244" s="8" t="n"/>
-    </row>
-    <row r="245">
-      <c r="A245" s="8" t="n"/>
-    </row>
-    <row r="246">
-      <c r="A246" s="8" t="n"/>
-    </row>
-    <row r="247">
-      <c r="A247" s="8" t="n"/>
-    </row>
-    <row r="248">
-      <c r="A248" s="8" t="n"/>
-    </row>
-    <row r="249">
-      <c r="A249" s="8" t="n"/>
-    </row>
-    <row r="250">
-      <c r="A250" s="8" t="n"/>
-    </row>
-    <row r="251">
-      <c r="A251" s="8" t="n"/>
-    </row>
-    <row r="252">
-      <c r="A252" s="8" t="n"/>
-    </row>
-    <row r="253">
-      <c r="A253" s="8" t="n"/>
-    </row>
-    <row r="254">
-      <c r="A254" s="8" t="n"/>
-    </row>
-    <row r="255">
-      <c r="A255" s="8" t="n"/>
-    </row>
-    <row r="256">
-      <c r="A256" s="8" t="n"/>
-    </row>
-    <row r="257">
-      <c r="A257" s="8" t="n"/>
-    </row>
-    <row r="258">
-      <c r="A258" s="8" t="n"/>
-    </row>
-    <row r="259">
-      <c r="A259" s="8" t="n"/>
-    </row>
-    <row r="260">
-      <c r="A260" s="8" t="n"/>
-    </row>
-    <row r="261">
-      <c r="A261" s="8" t="n"/>
-    </row>
-    <row r="262">
-      <c r="A262" s="8" t="n"/>
-    </row>
-    <row r="263">
-      <c r="A263" s="8" t="n"/>
-    </row>
-    <row r="264">
-      <c r="A264" s="8" t="n"/>
-    </row>
-    <row r="265">
-      <c r="A265" s="8" t="n"/>
-    </row>
-    <row r="266">
-      <c r="A266" s="8" t="n"/>
-    </row>
-    <row r="267">
-      <c r="A267" s="8" t="n"/>
-    </row>
-    <row r="268">
-      <c r="A268" s="8" t="n"/>
-    </row>
-    <row r="269">
-      <c r="A269" s="8" t="n"/>
-    </row>
-    <row r="270">
-      <c r="A270" s="8" t="n"/>
-    </row>
-    <row r="271">
-      <c r="A271" s="8" t="n"/>
-    </row>
-    <row r="272">
-      <c r="A272" s="8" t="n"/>
-    </row>
-    <row r="273">
-      <c r="A273" s="8" t="n"/>
-    </row>
-    <row r="274">
-      <c r="A274" s="8" t="n"/>
-    </row>
-    <row r="275">
-      <c r="A275" s="8" t="n"/>
-    </row>
-    <row r="276">
-      <c r="A276" s="8" t="n"/>
-    </row>
-    <row r="277">
-      <c r="A277" s="8" t="n"/>
-    </row>
-    <row r="278">
-      <c r="A278" s="8" t="n"/>
-    </row>
-    <row r="279">
-      <c r="A279" s="8" t="n"/>
-    </row>
-    <row r="280">
-      <c r="A280" s="8" t="n"/>
-    </row>
-    <row r="281">
-      <c r="A281" s="8" t="n"/>
-    </row>
-    <row r="282">
-      <c r="A282" s="8" t="n"/>
-    </row>
-    <row r="283">
-      <c r="A283" s="8" t="n"/>
-    </row>
-    <row r="284">
-      <c r="A284" s="8" t="n"/>
-    </row>
-    <row r="285">
-      <c r="A285" s="8" t="n"/>
-    </row>
-    <row r="286">
-      <c r="A286" s="8" t="n"/>
-    </row>
-    <row r="287">
-      <c r="A287" s="8" t="n"/>
-    </row>
-    <row r="288">
-      <c r="A288" s="8" t="n"/>
-    </row>
-    <row r="289">
-      <c r="A289" s="8" t="n"/>
-    </row>
-    <row r="290">
-      <c r="A290" s="8" t="n"/>
-    </row>
-    <row r="291">
-      <c r="A291" s="8" t="n"/>
-    </row>
-    <row r="292">
-      <c r="A292" s="8" t="n"/>
-    </row>
-    <row r="293">
-      <c r="A293" s="8" t="n"/>
-    </row>
-    <row r="294">
-      <c r="A294" s="8" t="n"/>
-    </row>
-    <row r="295">
-      <c r="A295" s="8" t="n"/>
-    </row>
-    <row r="296">
-      <c r="A296" s="8" t="n"/>
-    </row>
-    <row r="297">
-      <c r="A297" s="8" t="n"/>
-    </row>
-    <row r="298">
-      <c r="A298" s="8" t="n"/>
-    </row>
-    <row r="299">
-      <c r="A299" s="8" t="n"/>
-    </row>
-    <row r="300">
-      <c r="A300" s="8" t="n"/>
-    </row>
-    <row r="301">
-      <c r="A301" s="8" t="n"/>
-    </row>
-    <row r="302">
-      <c r="A302" s="8" t="n"/>
-    </row>
-    <row r="303">
-      <c r="A303" s="8" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="B4:B303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
-      <formula1>Lists!$Y$2:$Y$4</formula1>
-    </dataValidation>
-    <dataValidation sqref="E4:E303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Integer" error="请填非负整数。" type="whole" errorStyle="warning" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="002F75B5"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:Q803"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -14909,7 +12973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F75B5"/>
@@ -44740,7 +42804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F75B5"/>
@@ -45786,7 +43850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -47890,7 +45954,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007F7F7F"/>
@@ -48201,7 +46265,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007F7F7F"/>
@@ -48875,4 +46939,905 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00BBBBBB"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AF11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="44" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="40" customWidth="1" min="28" max="28"/>
+    <col width="37" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>yn</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>yn_nr</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>lang</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>ft_lang</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>consecutive</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>aetiology</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>ws_basis</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>presentation</t>
+        </is>
+      </c>
+      <c r="K1" s="17" t="inlineStr">
+        <is>
+          <t>deferred_reason</t>
+        </is>
+      </c>
+      <c r="L1" s="17" t="inlineStr">
+        <is>
+          <t>torsion_awaiting</t>
+        </is>
+      </c>
+      <c r="M1" s="17" t="inlineStr">
+        <is>
+          <t>perfusion</t>
+        </is>
+      </c>
+      <c r="N1" s="17" t="inlineStr">
+        <is>
+          <t>approach</t>
+        </is>
+      </c>
+      <c r="O1" s="17" t="inlineStr">
+        <is>
+          <t>viability</t>
+        </is>
+      </c>
+      <c r="P1" s="17" t="inlineStr">
+        <is>
+          <t>viab_basis</t>
+        </is>
+      </c>
+      <c r="Q1" s="17" t="inlineStr">
+        <is>
+          <t>procedure</t>
+        </is>
+      </c>
+      <c r="R1" s="17" t="inlineStr">
+        <is>
+          <t>fixation</t>
+        </is>
+      </c>
+      <c r="S1" s="17" t="inlineStr">
+        <is>
+          <t>reason_removed</t>
+        </is>
+      </c>
+      <c r="T1" s="17" t="inlineStr">
+        <is>
+          <t>status_fu</t>
+        </is>
+      </c>
+      <c r="U1" s="17" t="inlineStr">
+        <is>
+          <t>dur_category</t>
+        </is>
+      </c>
+      <c r="V1" s="17" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="W1" s="17" t="inlineStr">
+        <is>
+          <t>phrase</t>
+        </is>
+      </c>
+      <c r="X1" s="17" t="inlineStr">
+        <is>
+          <t>extractor</t>
+        </is>
+      </c>
+      <c r="Y1" s="17" t="inlineStr">
+        <is>
+          <t>ft_reviewer</t>
+        </is>
+      </c>
+      <c r="Z1" s="17" t="inlineStr">
+        <is>
+          <t>ft_decision</t>
+        </is>
+      </c>
+      <c r="AA1" s="17" t="inlineStr">
+        <is>
+          <t>ft_reason</t>
+        </is>
+      </c>
+      <c r="AB1" s="17" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="AC1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_final</t>
+        </is>
+      </c>
+      <c r="AD1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_received</t>
+        </is>
+      </c>
+      <c r="AE1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_delivery</t>
+        </is>
+      </c>
+      <c r="AF1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_reached</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Case report</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Congenital</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Imaging shows ectopic position or mobility</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Acute</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Family declined</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Viable</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Intraoperative</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Detorsion only</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Mesh</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Failure of fixation</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Preserved</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>&lt;=2 d</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>L other language</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Publisher or open access</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Not yet sent</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Case series</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Acquired</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Operation shows ectopic position or mobility</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Chronic or intermittent</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Observation advised</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Reduced</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Partially non-viable</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Histology</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Splenopexy</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Retroperitoneal or extraperitoneal pouch</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Surgeon's preference</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Partially preserved</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>3-7 d</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Less than 24 hours / a few hours / overnight</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>D no full text</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Library subscription</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Included with IPD</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Sent, no bounce</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cohort</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Imaging and operation</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Acute on chronic</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Elective operation scheduled</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Converted</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Non-viable</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Partial splenectomy +/- splenopexy</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Omental wrap</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Lost</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>8-30 d</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>weeks</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Consensus</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Consensus</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Pending IPD</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>E1 non-human</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Interlibrary loan or document delivery</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Narrative only (no individual data)</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Bounced</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Letter</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Named wandering spleen, no detail</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Asymptomatic</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Total splenectomy</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Direct suture</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>&gt;30 d</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>E2 not wandering spleen</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>CNKI or Wanfang</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Not eligible after check</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>No address found</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Review with new patients</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Torsion only, position not stated</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Mass only</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Autotransplantation</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Other (specify)</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>E3 adults only</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Contact author</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>No operation</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>E4 no original patient data</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>E5 not a formal article</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>Not obtained</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>E6 other</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>A aggregate data only</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>N age not confirmed under 18</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Record full-text calibration discussion outcome; guide v2026-10-19g (appendix data, ws_basis rule); release formal blank workbooks
Per-patient data in an online appendix counts as individual data; the two Chinese series
are Include and no longer IPD candidates. Formal FT_log blanks regenerated (v2026-10-19e).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction workbook - template (draft).xlsx
+++ b/Extraction workbook - template (draft).xlsx
@@ -559,7 +559,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>数据提取工作簿（模板，草稿）v2026-10-19d — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
+          <t>数据提取工作簿（模板，草稿）v2026-10-19e — 儿童游走脾系统综述（PROSPERO CRD420261520329）</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>仅 Include 时填（指南 D1 已决定：宽松加标记）</t>
+          <t>仅 Include 时填；Imaging and operation 只在影像和术中所见都写明脾异位或活动时选（指南 6.7）</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">

</xml_diff>